<commit_message>
Update OpenCart test cases
</commit_message>
<xml_diff>
--- a/OPEN CART TEST CASES.xlsx
+++ b/OPEN CART TEST CASES.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="8940" firstSheet="7" activeTab="10"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="8940"/>
   </bookViews>
   <sheets>
     <sheet name="Register" sheetId="1" r:id="rId1"/>
@@ -22,15 +22,15 @@
     <sheet name="Update Cart" sheetId="15" r:id="rId8"/>
     <sheet name="Product detail" sheetId="16" r:id="rId9"/>
     <sheet name="ATC from product page" sheetId="17" r:id="rId10"/>
-    <sheet name="Order confirmation" sheetId="19" r:id="rId11"/>
-    <sheet name="Checkout" sheetId="20" r:id="rId12"/>
+    <sheet name="Checkout" sheetId="20" r:id="rId11"/>
+    <sheet name="Order confirmation" sheetId="19" r:id="rId12"/>
   </sheets>
   <calcPr calcId="162913"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1123" uniqueCount="526">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1142" uniqueCount="536">
   <si>
     <t>TestCaseId</t>
   </si>
@@ -1626,9 +1626,6 @@
     <t>TC_CHK_009</t>
   </si>
   <si>
-    <t>TC_CHK_010</t>
-  </si>
-  <si>
     <t>Validate if checkout page loads correctly</t>
   </si>
   <si>
@@ -1637,9 +1634,6 @@
 3) Click Checkout button</t>
   </si>
   <si>
-    <t>Checkout page should load with billing details and order summary visible</t>
-  </si>
-  <si>
     <t>Validate if billing details are pre-filled for logged in user</t>
   </si>
   <si>
@@ -1671,9 +1665,6 @@
     <t>1) Proceed to checkout 
 2) Clear all billing fields 
 3) Click Continue</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Error messages shown for all mandatory billing fields</t>
   </si>
   <si>
     <t>Validate if invalid billing details give error</t>
@@ -1736,17 +1727,6 @@
     <t>Order placed successfully, redirected to order confirmation page</t>
   </si>
   <si>
-    <t>Validate if back button during checkout warns user or loses progress</t>
-  </si>
-  <si>
-    <t>1) Proceed to checkout 
-2) Fill some details 
-3) Click browser back button</t>
-  </si>
-  <si>
-    <t>User is warned about losing progress or is taken back safely without errors</t>
-  </si>
-  <si>
     <t>1) account created succesfully,user was redirected to success page
 2) continue on succes page directed to account page</t>
   </si>
@@ -1874,6 +1854,54 @@
   </si>
   <si>
     <t>Most product pages pass. Products with demo options (Apple Cinema, Canon EOS, HP LP3065) display irrelevant fields,Demo products display generic option fields — may be intentional demo behavior, not a real product bug.</t>
+  </si>
+  <si>
+    <t>Checkout page should loads succesfully</t>
+  </si>
+  <si>
+    <t>Order summary matches expected product/price. This section works independent of billing.</t>
+  </si>
+  <si>
+    <t>No Terms and Conditions checkbox is visible anywhere on the logged-in checkout page. Cannot verify enforcement. Blocked by TC_CHK_002/007.</t>
+  </si>
+  <si>
+    <t>For logged-in users, Personal Details and Shipping Address sections do not render, checkout skips directly to Payment Method. No billing fields present to verify pre-fill.</t>
+  </si>
+  <si>
+    <t>Cannot test, no billing fields are rendered for logged-in checkout, so "leave fields empty" cannot be attempted. Blocked by TC_CHK_002.</t>
+  </si>
+  <si>
+    <t>Cannot test. same as above, no billing fields exist to enter invalid data into. Blocked by TC_CHK_002.</t>
+  </si>
+  <si>
+    <t>Cannot test, no shipping method selection UI is shown at all for logged-in checkout. Blocked by TC_CHK_002.</t>
+  </si>
+  <si>
+    <t>Error messages shown for all mandatory billing fields</t>
+  </si>
+  <si>
+    <t>Payment Method dropdown shows "No Payment options are available. Please contact us for assistance!", no options can be selected.</t>
+  </si>
+  <si>
+    <t>Order cannot be placed, Confirm Order cannot succeed without a selected payment method as the button is unclickable.</t>
+  </si>
+  <si>
+    <t>Cannot verify, checkout process cannot be completed due to no payment metods available at TC_CHK_007. No order confirmation page reached. Blocked by TC_CHK_007.</t>
+  </si>
+  <si>
+    <t>Blocked by TC_CHK_007</t>
+  </si>
+  <si>
+    <t>Cannot verify, no order placed, so nothing to check in order history. Blocked by TC_CHK_007.</t>
+  </si>
+  <si>
+    <t>Cannot verify, same blocker, checkout cannot be completed to reach confirmation page. Blocked by TC_CHK_007.</t>
+  </si>
+  <si>
+    <t>Cannot verify, checkout cannot be completed, no order placed, no confirmation email triggered. Blocked by TC_CHK_007.</t>
+  </si>
+  <si>
+    <t>Cannot verify, no confirmation page reached to test Continue button. Blocked by TC_CHK_007.</t>
   </si>
 </sst>
 </file>
@@ -2098,16 +2126,16 @@
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -2341,18 +2369,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="21" x14ac:dyDescent="0.35">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="16" t="s">
         <v>12</v>
       </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="13"/>
-      <c r="D1" s="13"/>
-      <c r="E1" s="13"/>
-      <c r="F1" s="13"/>
-      <c r="G1" s="13"/>
-      <c r="H1" s="13"/>
-      <c r="I1" s="13"/>
-      <c r="J1" s="13"/>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="17"/>
+      <c r="F1" s="17"/>
+      <c r="G1" s="17"/>
+      <c r="H1" s="17"/>
+      <c r="I1" s="17"/>
+      <c r="J1" s="17"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
@@ -2402,7 +2430,7 @@
       <c r="E3" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="F3" s="14" t="s">
+      <c r="F3" s="12" t="s">
         <v>39</v>
       </c>
       <c r="G3" s="8" t="s">
@@ -2412,7 +2440,7 @@
         <v>69</v>
       </c>
       <c r="I3" s="4" t="s">
-        <v>485</v>
+        <v>479</v>
       </c>
       <c r="J3" s="5" t="s">
         <v>11</v>
@@ -2434,7 +2462,7 @@
       <c r="E4" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="F4" s="14" t="s">
+      <c r="F4" s="12" t="s">
         <v>41</v>
       </c>
       <c r="G4" s="8" t="s">
@@ -2447,7 +2475,7 @@
         <v>42</v>
       </c>
       <c r="J4" s="5" t="s">
-        <v>486</v>
+        <v>480</v>
       </c>
     </row>
     <row r="5" spans="1:10" ht="61.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2466,7 +2494,7 @@
       <c r="E5" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="F5" s="14" t="s">
+      <c r="F5" s="12" t="s">
         <v>43</v>
       </c>
       <c r="G5" s="8" t="s">
@@ -2476,10 +2504,10 @@
         <v>45</v>
       </c>
       <c r="I5" s="4" t="s">
-        <v>520</v>
-      </c>
-      <c r="J5" s="16" t="s">
-        <v>521</v>
+        <v>514</v>
+      </c>
+      <c r="J5" s="14" t="s">
+        <v>515</v>
       </c>
     </row>
     <row r="6" spans="1:10" ht="52.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2498,7 +2526,7 @@
       <c r="E6" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="F6" s="14" t="s">
+      <c r="F6" s="12" t="s">
         <v>81</v>
       </c>
       <c r="G6" s="8" t="s">
@@ -2508,10 +2536,10 @@
         <v>47</v>
       </c>
       <c r="I6" s="4" t="s">
-        <v>488</v>
+        <v>482</v>
       </c>
       <c r="J6" s="5" t="s">
-        <v>486</v>
+        <v>480</v>
       </c>
     </row>
     <row r="7" spans="1:10" ht="125.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -2530,7 +2558,7 @@
       <c r="E7" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="F7" s="14" t="s">
+      <c r="F7" s="12" t="s">
         <v>73</v>
       </c>
       <c r="G7" s="6" t="s">
@@ -2540,10 +2568,10 @@
         <v>48</v>
       </c>
       <c r="I7" s="4" t="s">
-        <v>488</v>
+        <v>482</v>
       </c>
       <c r="J7" s="5" t="s">
-        <v>486</v>
+        <v>480</v>
       </c>
     </row>
     <row r="8" spans="1:10" ht="98.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -2562,7 +2590,7 @@
       <c r="E8" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="F8" s="14" t="s">
+      <c r="F8" s="12" t="s">
         <v>74</v>
       </c>
       <c r="G8" s="8" t="s">
@@ -2572,10 +2600,10 @@
         <v>51</v>
       </c>
       <c r="I8" s="4" t="s">
-        <v>488</v>
+        <v>482</v>
       </c>
       <c r="J8" s="5" t="s">
-        <v>486</v>
+        <v>480</v>
       </c>
     </row>
     <row r="9" spans="1:10" ht="82.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2594,7 +2622,7 @@
       <c r="E9" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="F9" s="14" t="s">
+      <c r="F9" s="12" t="s">
         <v>75</v>
       </c>
       <c r="G9" s="8" t="s">
@@ -2604,10 +2632,10 @@
         <v>56</v>
       </c>
       <c r="I9" s="4" t="s">
-        <v>489</v>
-      </c>
-      <c r="J9" s="15" t="s">
-        <v>487</v>
+        <v>483</v>
+      </c>
+      <c r="J9" s="13" t="s">
+        <v>481</v>
       </c>
     </row>
     <row r="10" spans="1:10" ht="82.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2626,7 +2654,7 @@
       <c r="E10" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="F10" s="14" t="s">
+      <c r="F10" s="12" t="s">
         <v>82</v>
       </c>
       <c r="G10" s="8" t="s">
@@ -2636,10 +2664,10 @@
         <v>57</v>
       </c>
       <c r="I10" s="4" t="s">
-        <v>488</v>
+        <v>482</v>
       </c>
       <c r="J10" s="5" t="s">
-        <v>486</v>
+        <v>480</v>
       </c>
     </row>
     <row r="11" spans="1:10" ht="85.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2658,7 +2686,7 @@
       <c r="E11" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="F11" s="14" t="s">
+      <c r="F11" s="12" t="s">
         <v>76</v>
       </c>
       <c r="G11" s="8" t="s">
@@ -2668,10 +2696,10 @@
         <v>59</v>
       </c>
       <c r="I11" s="4" t="s">
-        <v>488</v>
+        <v>482</v>
       </c>
       <c r="J11" s="5" t="s">
-        <v>486</v>
+        <v>480</v>
       </c>
     </row>
     <row r="12" spans="1:10" ht="88.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2690,7 +2718,7 @@
       <c r="E12" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="F12" s="14" t="s">
+      <c r="F12" s="12" t="s">
         <v>77</v>
       </c>
       <c r="G12" s="8" t="s">
@@ -2700,10 +2728,10 @@
         <v>61</v>
       </c>
       <c r="I12" s="4" t="s">
-        <v>490</v>
-      </c>
-      <c r="J12" s="15" t="s">
-        <v>487</v>
+        <v>484</v>
+      </c>
+      <c r="J12" s="13" t="s">
+        <v>481</v>
       </c>
     </row>
     <row r="13" spans="1:10" ht="88.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2722,7 +2750,7 @@
       <c r="E13" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="F13" s="14" t="s">
+      <c r="F13" s="12" t="s">
         <v>78</v>
       </c>
       <c r="G13" s="8" t="s">
@@ -2732,10 +2760,10 @@
         <v>63</v>
       </c>
       <c r="I13" s="4" t="s">
-        <v>488</v>
+        <v>482</v>
       </c>
       <c r="J13" s="5" t="s">
-        <v>486</v>
+        <v>480</v>
       </c>
     </row>
     <row r="14" spans="1:10" ht="73.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2754,7 +2782,7 @@
       <c r="E14" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="F14" s="14" t="s">
+      <c r="F14" s="12" t="s">
         <v>79</v>
       </c>
       <c r="G14" s="8" t="s">
@@ -2764,10 +2792,10 @@
         <v>65</v>
       </c>
       <c r="I14" s="4" t="s">
-        <v>488</v>
+        <v>482</v>
       </c>
       <c r="J14" s="5" t="s">
-        <v>486</v>
+        <v>480</v>
       </c>
     </row>
     <row r="15" spans="1:10" ht="75" customHeight="1" x14ac:dyDescent="0.25">
@@ -2786,7 +2814,7 @@
       <c r="E15" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="F15" s="14" t="s">
+      <c r="F15" s="12" t="s">
         <v>84</v>
       </c>
       <c r="G15" s="8" t="s">
@@ -2796,7 +2824,7 @@
         <v>66</v>
       </c>
       <c r="I15" s="4" t="s">
-        <v>488</v>
+        <v>482</v>
       </c>
       <c r="J15" s="5" t="s">
         <v>11</v>
@@ -2818,7 +2846,7 @@
       <c r="E16" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="F16" s="14" t="s">
+      <c r="F16" s="12" t="s">
         <v>80</v>
       </c>
       <c r="G16" s="8" t="s">
@@ -2828,7 +2856,7 @@
         <v>68</v>
       </c>
       <c r="I16" s="4" t="s">
-        <v>488</v>
+        <v>482</v>
       </c>
       <c r="J16" s="5" t="s">
         <v>11</v>
@@ -2850,7 +2878,7 @@
       <c r="E17" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="F17" s="14" t="s">
+      <c r="F17" s="12" t="s">
         <v>87</v>
       </c>
       <c r="G17" s="8" t="s">
@@ -2860,7 +2888,7 @@
         <v>90</v>
       </c>
       <c r="I17" s="4" t="s">
-        <v>488</v>
+        <v>482</v>
       </c>
       <c r="J17" s="5" t="s">
         <v>11</v>
@@ -2882,7 +2910,7 @@
       <c r="E18" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="F18" s="14" t="s">
+      <c r="F18" s="12" t="s">
         <v>92</v>
       </c>
       <c r="G18" s="8" t="s">
@@ -2892,7 +2920,7 @@
         <v>94</v>
       </c>
       <c r="I18" s="4" t="s">
-        <v>488</v>
+        <v>482</v>
       </c>
       <c r="J18" s="5" t="s">
         <v>11</v>
@@ -2914,7 +2942,7 @@
       <c r="E19" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="F19" s="14" t="s">
+      <c r="F19" s="12" t="s">
         <v>96</v>
       </c>
       <c r="G19" s="8" t="s">
@@ -2924,10 +2952,10 @@
         <v>98</v>
       </c>
       <c r="I19" s="4" t="s">
-        <v>491</v>
+        <v>485</v>
       </c>
       <c r="J19" s="5" t="s">
-        <v>486</v>
+        <v>480</v>
       </c>
     </row>
     <row r="20" spans="1:10" ht="90.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -2936,7 +2964,7 @@
       <c r="C20" s="2"/>
       <c r="D20" s="4"/>
       <c r="E20" s="4"/>
-      <c r="F20" s="14"/>
+      <c r="F20" s="12"/>
       <c r="G20" s="8"/>
       <c r="H20" s="4"/>
       <c r="I20" s="4"/>
@@ -2948,7 +2976,7 @@
       <c r="C21" s="2"/>
       <c r="D21" s="4"/>
       <c r="E21" s="4"/>
-      <c r="F21" s="14"/>
+      <c r="F21" s="12"/>
       <c r="G21" s="8"/>
       <c r="H21" s="4"/>
       <c r="I21" s="4"/>
@@ -2960,7 +2988,7 @@
       <c r="C22" s="2"/>
       <c r="D22" s="4"/>
       <c r="E22" s="4"/>
-      <c r="F22" s="14"/>
+      <c r="F22" s="12"/>
       <c r="G22" s="8"/>
       <c r="H22" s="4"/>
       <c r="I22" s="4"/>
@@ -3982,18 +4010,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="21" x14ac:dyDescent="0.35">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="16" t="s">
         <v>379</v>
       </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="13"/>
-      <c r="D1" s="13"/>
-      <c r="E1" s="13"/>
-      <c r="F1" s="13"/>
-      <c r="G1" s="13"/>
-      <c r="H1" s="13"/>
-      <c r="I1" s="13"/>
-      <c r="J1" s="13"/>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="17"/>
+      <c r="F1" s="17"/>
+      <c r="G1" s="17"/>
+      <c r="H1" s="17"/>
+      <c r="I1" s="17"/>
+      <c r="J1" s="17"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
@@ -4043,7 +4071,7 @@
       <c r="E3" s="4" t="s">
         <v>381</v>
       </c>
-      <c r="F3" s="14" t="s">
+      <c r="F3" s="12" t="s">
         <v>383</v>
       </c>
       <c r="G3" s="8" t="s">
@@ -4053,7 +4081,7 @@
         <v>389</v>
       </c>
       <c r="I3" s="4" t="s">
-        <v>488</v>
+        <v>482</v>
       </c>
       <c r="J3" s="5" t="s">
         <v>11</v>
@@ -4075,7 +4103,7 @@
       <c r="E4" s="4" t="s">
         <v>381</v>
       </c>
-      <c r="F4" s="14" t="s">
+      <c r="F4" s="12" t="s">
         <v>386</v>
       </c>
       <c r="G4" s="8" t="s">
@@ -4085,7 +4113,7 @@
         <v>388</v>
       </c>
       <c r="I4" s="4" t="s">
-        <v>488</v>
+        <v>482</v>
       </c>
       <c r="J4" s="5" t="s">
         <v>11</v>
@@ -4107,7 +4135,7 @@
       <c r="E5" s="4" t="s">
         <v>381</v>
       </c>
-      <c r="F5" s="14" t="s">
+      <c r="F5" s="12" t="s">
         <v>391</v>
       </c>
       <c r="G5" s="8" t="s">
@@ -4117,10 +4145,10 @@
         <v>393</v>
       </c>
       <c r="I5" s="4" t="s">
-        <v>506</v>
-      </c>
-      <c r="J5" s="15" t="s">
-        <v>494</v>
+        <v>500</v>
+      </c>
+      <c r="J5" s="13" t="s">
+        <v>488</v>
       </c>
     </row>
     <row r="6" spans="1:10" ht="111" customHeight="1" x14ac:dyDescent="0.25">
@@ -4139,7 +4167,7 @@
       <c r="E6" s="4" t="s">
         <v>381</v>
       </c>
-      <c r="F6" s="14" t="s">
+      <c r="F6" s="12" t="s">
         <v>395</v>
       </c>
       <c r="G6" s="8" t="s">
@@ -4149,10 +4177,10 @@
         <v>397</v>
       </c>
       <c r="I6" s="4" t="s">
-        <v>507</v>
-      </c>
-      <c r="J6" s="15" t="s">
-        <v>494</v>
+        <v>501</v>
+      </c>
+      <c r="J6" s="13" t="s">
+        <v>488</v>
       </c>
     </row>
     <row r="7" spans="1:10" ht="81" customHeight="1" x14ac:dyDescent="0.25">
@@ -4171,7 +4199,7 @@
       <c r="E7" s="4" t="s">
         <v>381</v>
       </c>
-      <c r="F7" s="14" t="s">
+      <c r="F7" s="12" t="s">
         <v>399</v>
       </c>
       <c r="G7" s="8" t="s">
@@ -4181,10 +4209,10 @@
         <v>401</v>
       </c>
       <c r="I7" s="4" t="s">
-        <v>508</v>
-      </c>
-      <c r="J7" s="15" t="s">
-        <v>494</v>
+        <v>502</v>
+      </c>
+      <c r="J7" s="13" t="s">
+        <v>488</v>
       </c>
     </row>
     <row r="8" spans="1:10" ht="76.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -4203,7 +4231,7 @@
       <c r="E8" s="4" t="s">
         <v>381</v>
       </c>
-      <c r="F8" s="14" t="s">
+      <c r="F8" s="12" t="s">
         <v>403</v>
       </c>
       <c r="G8" s="6" t="s">
@@ -4213,7 +4241,7 @@
         <v>404</v>
       </c>
       <c r="I8" s="4" t="s">
-        <v>488</v>
+        <v>482</v>
       </c>
       <c r="J8" s="5" t="s">
         <v>11</v>
@@ -4235,7 +4263,7 @@
       <c r="E9" s="4" t="s">
         <v>381</v>
       </c>
-      <c r="F9" s="14" t="s">
+      <c r="F9" s="12" t="s">
         <v>406</v>
       </c>
       <c r="G9" s="8" t="s">
@@ -4245,7 +4273,7 @@
         <v>407</v>
       </c>
       <c r="I9" s="4" t="s">
-        <v>488</v>
+        <v>482</v>
       </c>
       <c r="J9" s="5" t="s">
         <v>11</v>
@@ -4267,7 +4295,7 @@
       <c r="E10" s="4" t="s">
         <v>381</v>
       </c>
-      <c r="F10" s="14" t="s">
+      <c r="F10" s="12" t="s">
         <v>410</v>
       </c>
       <c r="G10" s="8" t="s">
@@ -4277,7 +4305,7 @@
         <v>411</v>
       </c>
       <c r="I10" s="4" t="s">
-        <v>488</v>
+        <v>482</v>
       </c>
       <c r="J10" s="5" t="s">
         <v>11</v>
@@ -4294,25 +4322,25 @@
         <v>10</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>509</v>
+        <v>503</v>
       </c>
       <c r="E11" s="4" t="s">
         <v>381</v>
       </c>
-      <c r="F11" s="14" t="s">
-        <v>510</v>
+      <c r="F11" s="12" t="s">
+        <v>504</v>
       </c>
       <c r="G11" s="8" t="s">
-        <v>511</v>
+        <v>505</v>
       </c>
       <c r="H11" s="4" t="s">
-        <v>512</v>
+        <v>506</v>
       </c>
       <c r="I11" s="4" t="s">
-        <v>513</v>
-      </c>
-      <c r="J11" s="15" t="s">
-        <v>494</v>
+        <v>507</v>
+      </c>
+      <c r="J11" s="13" t="s">
+        <v>488</v>
       </c>
     </row>
     <row r="12" spans="1:10" ht="85.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -4321,7 +4349,7 @@
       <c r="C12" s="2"/>
       <c r="D12" s="4"/>
       <c r="E12" s="4"/>
-      <c r="F12" s="14"/>
+      <c r="F12" s="12"/>
       <c r="G12" s="8"/>
       <c r="H12" s="4"/>
       <c r="I12" s="4"/>
@@ -4333,7 +4361,7 @@
       <c r="C13" s="2"/>
       <c r="D13" s="4"/>
       <c r="E13" s="4"/>
-      <c r="F13" s="14"/>
+      <c r="F13" s="12"/>
       <c r="G13" s="8"/>
       <c r="H13" s="4"/>
       <c r="I13" s="4"/>
@@ -4345,7 +4373,7 @@
       <c r="C14" s="2"/>
       <c r="D14" s="4"/>
       <c r="E14" s="4"/>
-      <c r="F14" s="14"/>
+      <c r="F14" s="12"/>
       <c r="G14" s="8"/>
       <c r="H14" s="4"/>
       <c r="I14" s="4"/>
@@ -4357,7 +4385,7 @@
       <c r="C15" s="2"/>
       <c r="D15" s="4"/>
       <c r="E15" s="4"/>
-      <c r="F15" s="14"/>
+      <c r="F15" s="12"/>
       <c r="G15" s="8"/>
       <c r="H15" s="4"/>
       <c r="I15" s="4"/>
@@ -4369,7 +4397,7 @@
       <c r="C16" s="2"/>
       <c r="D16" s="4"/>
       <c r="E16" s="4"/>
-      <c r="F16" s="14"/>
+      <c r="F16" s="12"/>
       <c r="G16" s="8"/>
       <c r="H16" s="4"/>
       <c r="I16" s="4"/>
@@ -4381,7 +4409,7 @@
       <c r="C17" s="2"/>
       <c r="D17" s="4"/>
       <c r="E17" s="4"/>
-      <c r="F17" s="14"/>
+      <c r="F17" s="12"/>
       <c r="G17" s="8"/>
       <c r="H17" s="4"/>
       <c r="I17" s="4"/>
@@ -4393,7 +4421,7 @@
       <c r="C18" s="2"/>
       <c r="D18" s="4"/>
       <c r="E18" s="4"/>
-      <c r="F18" s="14"/>
+      <c r="F18" s="12"/>
       <c r="G18" s="8"/>
       <c r="H18" s="4"/>
       <c r="I18" s="4"/>
@@ -4405,7 +4433,7 @@
       <c r="C19" s="2"/>
       <c r="D19" s="4"/>
       <c r="E19" s="4"/>
-      <c r="F19" s="14"/>
+      <c r="F19" s="12"/>
       <c r="G19" s="8"/>
       <c r="H19" s="4"/>
       <c r="I19" s="4"/>
@@ -4417,7 +4445,7 @@
       <c r="C20" s="2"/>
       <c r="D20" s="4"/>
       <c r="E20" s="4"/>
-      <c r="F20" s="14"/>
+      <c r="F20" s="12"/>
       <c r="G20" s="8"/>
       <c r="H20" s="4"/>
       <c r="I20" s="4"/>
@@ -4429,7 +4457,7 @@
       <c r="C21" s="2"/>
       <c r="D21" s="4"/>
       <c r="E21" s="4"/>
-      <c r="F21" s="14"/>
+      <c r="F21" s="12"/>
       <c r="G21" s="8"/>
       <c r="H21" s="4"/>
       <c r="I21" s="4"/>
@@ -4441,7 +4469,7 @@
       <c r="C22" s="2"/>
       <c r="D22" s="4"/>
       <c r="E22" s="4"/>
-      <c r="F22" s="14"/>
+      <c r="F22" s="12"/>
       <c r="G22" s="8"/>
       <c r="H22" s="4"/>
       <c r="I22" s="4"/>
@@ -4453,7 +4481,7 @@
       <c r="C23" s="2"/>
       <c r="D23" s="4"/>
       <c r="E23" s="4"/>
-      <c r="F23" s="14"/>
+      <c r="F23" s="12"/>
       <c r="G23" s="8"/>
       <c r="H23" s="4"/>
       <c r="I23" s="4"/>
@@ -5458,7 +5486,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J1000"/>
+  <dimension ref="A1:J999"/>
   <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15.85546875" customWidth="1"/>
@@ -5469,24 +5497,24 @@
     <col min="6" max="6" width="34.5703125" style="11" customWidth="1"/>
     <col min="7" max="7" width="22.85546875" customWidth="1"/>
     <col min="8" max="8" width="23.7109375" customWidth="1"/>
-    <col min="9" max="9" width="17.140625" customWidth="1"/>
+    <col min="9" max="9" width="20.140625" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="9.28515625" customWidth="1"/>
     <col min="11" max="26" width="8.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="21" x14ac:dyDescent="0.35">
-      <c r="A1" s="12" t="s">
-        <v>412</v>
-      </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="13"/>
-      <c r="D1" s="13"/>
-      <c r="E1" s="13"/>
-      <c r="F1" s="13"/>
-      <c r="G1" s="13"/>
-      <c r="H1" s="13"/>
-      <c r="I1" s="13"/>
-      <c r="J1" s="13"/>
+      <c r="A1" s="16" t="s">
+        <v>440</v>
+      </c>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="17"/>
+      <c r="F1" s="17"/>
+      <c r="G1" s="17"/>
+      <c r="H1" s="17"/>
+      <c r="I1" s="17"/>
+      <c r="J1" s="17"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
@@ -5522,217 +5550,299 @@
     </row>
     <row r="3" spans="1:10" ht="88.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>414</v>
+        <v>441</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>413</v>
+        <v>447</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>10</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>421</v>
+        <v>452</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>420</v>
-      </c>
-      <c r="F3" s="14" t="s">
-        <v>427</v>
+        <v>448</v>
+      </c>
+      <c r="F3" s="12" t="s">
+        <v>453</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>258</v>
+        <v>50</v>
       </c>
       <c r="H3" s="4" t="s">
-        <v>434</v>
-      </c>
-      <c r="I3" s="4"/>
+        <v>520</v>
+      </c>
+      <c r="I3" s="4" t="s">
+        <v>482</v>
+      </c>
       <c r="J3" s="5" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="4" spans="1:10" ht="89.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:10" ht="102.75" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>415</v>
+        <v>442</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>413</v>
+        <v>447</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>10</v>
+        <v>40</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>422</v>
+        <v>454</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>420</v>
-      </c>
-      <c r="F4" s="14" t="s">
-        <v>428</v>
+        <v>448</v>
+      </c>
+      <c r="F4" s="12" t="s">
+        <v>455</v>
       </c>
       <c r="G4" s="8" t="s">
         <v>50</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>435</v>
-      </c>
-      <c r="I4" s="4"/>
-      <c r="J4" s="5"/>
-    </row>
-    <row r="5" spans="1:10" ht="85.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>456</v>
+      </c>
+      <c r="I4" s="4" t="s">
+        <v>523</v>
+      </c>
+      <c r="J4" s="13" t="s">
+        <v>488</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" ht="80.25" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>416</v>
+        <v>443</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>413</v>
+        <v>447</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>10</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>423</v>
+        <v>457</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>420</v>
-      </c>
-      <c r="F5" s="14" t="s">
-        <v>429</v>
+        <v>448</v>
+      </c>
+      <c r="F5" s="12" t="s">
+        <v>458</v>
       </c>
       <c r="G5" s="8" t="s">
-        <v>384</v>
+        <v>459</v>
       </c>
       <c r="H5" s="4" t="s">
-        <v>436</v>
-      </c>
-      <c r="I5" s="4"/>
-      <c r="J5" s="5"/>
-    </row>
-    <row r="6" spans="1:10" ht="79.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>460</v>
+      </c>
+      <c r="I5" s="4" t="s">
+        <v>521</v>
+      </c>
+      <c r="J5" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" ht="91.5" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>417</v>
+        <v>444</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>413</v>
+        <v>447</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>40</v>
+        <v>10</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>424</v>
+        <v>461</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>420</v>
-      </c>
-      <c r="F6" s="14" t="s">
-        <v>430</v>
+        <v>448</v>
+      </c>
+      <c r="F6" s="12" t="s">
+        <v>462</v>
       </c>
       <c r="G6" s="8" t="s">
-        <v>433</v>
+        <v>50</v>
       </c>
       <c r="H6" s="4" t="s">
-        <v>437</v>
-      </c>
-      <c r="I6" s="4"/>
-      <c r="J6" s="5"/>
+        <v>527</v>
+      </c>
+      <c r="I6" s="4" t="s">
+        <v>524</v>
+      </c>
+      <c r="J6" s="14" t="s">
+        <v>516</v>
+      </c>
     </row>
     <row r="7" spans="1:10" ht="81" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>418</v>
+        <v>445</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>413</v>
+        <v>447</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>40</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>425</v>
+        <v>463</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>420</v>
-      </c>
-      <c r="F7" s="14" t="s">
-        <v>431</v>
+        <v>448</v>
+      </c>
+      <c r="F7" s="12" t="s">
+        <v>464</v>
       </c>
       <c r="G7" s="8" t="s">
-        <v>50</v>
+        <v>465</v>
       </c>
       <c r="H7" s="4" t="s">
-        <v>438</v>
-      </c>
-      <c r="I7" s="4"/>
-      <c r="J7" s="5"/>
-    </row>
-    <row r="8" spans="1:10" ht="76.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>466</v>
+      </c>
+      <c r="I7" s="4" t="s">
+        <v>525</v>
+      </c>
+      <c r="J7" s="14" t="s">
+        <v>516</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" ht="80.25" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>419</v>
+        <v>446</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>413</v>
+        <v>447</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>40</v>
+        <v>10</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>426</v>
+        <v>467</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>420</v>
-      </c>
-      <c r="F8" s="14" t="s">
-        <v>432</v>
+        <v>448</v>
+      </c>
+      <c r="F8" s="12" t="s">
+        <v>468</v>
       </c>
       <c r="G8" s="6" t="s">
         <v>50</v>
       </c>
       <c r="H8" s="4" t="s">
-        <v>439</v>
-      </c>
-      <c r="I8" s="4"/>
-      <c r="J8" s="5"/>
-    </row>
-    <row r="9" spans="1:10" ht="78" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="2"/>
-      <c r="B9" s="2"/>
-      <c r="C9" s="2"/>
-      <c r="D9" s="4"/>
-      <c r="E9" s="4"/>
-      <c r="F9" s="14"/>
-      <c r="G9" s="8"/>
-      <c r="H9" s="4"/>
-      <c r="I9" s="4"/>
-      <c r="J9" s="5"/>
-    </row>
-    <row r="10" spans="1:10" ht="68.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="2"/>
-      <c r="B10" s="2"/>
-      <c r="C10" s="2"/>
-      <c r="D10" s="4"/>
-      <c r="E10" s="4"/>
-      <c r="F10" s="14"/>
-      <c r="G10" s="8"/>
-      <c r="H10" s="4"/>
-      <c r="I10" s="4"/>
-      <c r="J10" s="5"/>
-    </row>
-    <row r="11" spans="1:10" ht="82.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="2"/>
-      <c r="B11" s="2"/>
-      <c r="C11" s="2"/>
-      <c r="D11" s="4"/>
-      <c r="E11" s="4"/>
-      <c r="F11" s="14"/>
-      <c r="G11" s="8"/>
-      <c r="H11" s="4"/>
-      <c r="I11" s="4"/>
-      <c r="J11" s="5"/>
-    </row>
-    <row r="12" spans="1:10" ht="85.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>469</v>
+      </c>
+      <c r="I8" s="4" t="s">
+        <v>526</v>
+      </c>
+      <c r="J8" s="14" t="s">
+        <v>516</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" ht="102.75" x14ac:dyDescent="0.25">
+      <c r="A9" s="2" t="s">
+        <v>449</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>447</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>470</v>
+      </c>
+      <c r="E9" s="4" t="s">
+        <v>448</v>
+      </c>
+      <c r="F9" s="12" t="s">
+        <v>471</v>
+      </c>
+      <c r="G9" s="8" t="s">
+        <v>50</v>
+      </c>
+      <c r="H9" s="4" t="s">
+        <v>472</v>
+      </c>
+      <c r="I9" s="4" t="s">
+        <v>528</v>
+      </c>
+      <c r="J9" s="13" t="s">
+        <v>488</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" ht="102.75" x14ac:dyDescent="0.25">
+      <c r="A10" s="2" t="s">
+        <v>450</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>447</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>473</v>
+      </c>
+      <c r="E10" s="4" t="s">
+        <v>448</v>
+      </c>
+      <c r="F10" s="12" t="s">
+        <v>474</v>
+      </c>
+      <c r="G10" s="8" t="s">
+        <v>50</v>
+      </c>
+      <c r="H10" s="4" t="s">
+        <v>475</v>
+      </c>
+      <c r="I10" s="4" t="s">
+        <v>522</v>
+      </c>
+      <c r="J10" s="14" t="s">
+        <v>516</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" ht="80.25" x14ac:dyDescent="0.25">
+      <c r="A11" s="2" t="s">
+        <v>451</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>447</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D11" s="4" t="s">
+        <v>476</v>
+      </c>
+      <c r="E11" s="4" t="s">
+        <v>448</v>
+      </c>
+      <c r="F11" s="12" t="s">
+        <v>477</v>
+      </c>
+      <c r="G11" s="8" t="s">
+        <v>50</v>
+      </c>
+      <c r="H11" s="4" t="s">
+        <v>478</v>
+      </c>
+      <c r="I11" s="4" t="s">
+        <v>529</v>
+      </c>
+      <c r="J11" s="14" t="s">
+        <v>516</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" ht="88.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="2"/>
       <c r="B12" s="2"/>
       <c r="C12" s="2"/>
       <c r="D12" s="4"/>
       <c r="E12" s="4"/>
-      <c r="F12" s="14"/>
+      <c r="F12" s="12"/>
       <c r="G12" s="8"/>
       <c r="H12" s="4"/>
       <c r="I12" s="4"/>
@@ -5744,103 +5854,103 @@
       <c r="C13" s="2"/>
       <c r="D13" s="4"/>
       <c r="E13" s="4"/>
-      <c r="F13" s="14"/>
+      <c r="F13" s="12"/>
       <c r="G13" s="8"/>
       <c r="H13" s="4"/>
       <c r="I13" s="4"/>
       <c r="J13" s="5"/>
     </row>
-    <row r="14" spans="1:10" ht="88.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:10" ht="73.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="2"/>
       <c r="B14" s="2"/>
       <c r="C14" s="2"/>
       <c r="D14" s="4"/>
       <c r="E14" s="4"/>
-      <c r="F14" s="14"/>
+      <c r="F14" s="12"/>
       <c r="G14" s="8"/>
       <c r="H14" s="4"/>
       <c r="I14" s="4"/>
       <c r="J14" s="5"/>
     </row>
-    <row r="15" spans="1:10" ht="73.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:10" ht="75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="2"/>
       <c r="B15" s="2"/>
       <c r="C15" s="2"/>
       <c r="D15" s="4"/>
       <c r="E15" s="4"/>
-      <c r="F15" s="14"/>
+      <c r="F15" s="12"/>
       <c r="G15" s="8"/>
       <c r="H15" s="4"/>
       <c r="I15" s="4"/>
       <c r="J15" s="5"/>
     </row>
-    <row r="16" spans="1:10" ht="75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:10" ht="66.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="2"/>
       <c r="B16" s="2"/>
       <c r="C16" s="2"/>
       <c r="D16" s="4"/>
       <c r="E16" s="4"/>
-      <c r="F16" s="14"/>
+      <c r="F16" s="12"/>
       <c r="G16" s="8"/>
       <c r="H16" s="4"/>
       <c r="I16" s="4"/>
       <c r="J16" s="5"/>
     </row>
-    <row r="17" spans="1:10" ht="66.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:10" ht="71.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="2"/>
       <c r="B17" s="2"/>
       <c r="C17" s="2"/>
       <c r="D17" s="4"/>
       <c r="E17" s="4"/>
-      <c r="F17" s="14"/>
+      <c r="F17" s="12"/>
       <c r="G17" s="8"/>
       <c r="H17" s="4"/>
       <c r="I17" s="4"/>
       <c r="J17" s="5"/>
     </row>
-    <row r="18" spans="1:10" ht="71.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:10" ht="91.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="2"/>
       <c r="B18" s="2"/>
       <c r="C18" s="2"/>
       <c r="D18" s="4"/>
       <c r="E18" s="4"/>
-      <c r="F18" s="14"/>
+      <c r="F18" s="12"/>
       <c r="G18" s="8"/>
       <c r="H18" s="4"/>
       <c r="I18" s="4"/>
       <c r="J18" s="5"/>
     </row>
-    <row r="19" spans="1:10" ht="91.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:10" ht="80.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="2"/>
       <c r="B19" s="2"/>
       <c r="C19" s="2"/>
       <c r="D19" s="4"/>
       <c r="E19" s="4"/>
-      <c r="F19" s="14"/>
+      <c r="F19" s="12"/>
       <c r="G19" s="8"/>
       <c r="H19" s="4"/>
       <c r="I19" s="4"/>
       <c r="J19" s="5"/>
     </row>
-    <row r="20" spans="1:10" ht="80.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:10" ht="90.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="2"/>
       <c r="B20" s="2"/>
       <c r="C20" s="2"/>
       <c r="D20" s="4"/>
       <c r="E20" s="4"/>
-      <c r="F20" s="14"/>
+      <c r="F20" s="12"/>
       <c r="G20" s="8"/>
       <c r="H20" s="4"/>
       <c r="I20" s="4"/>
       <c r="J20" s="5"/>
     </row>
-    <row r="21" spans="1:10" ht="90.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="2"/>
       <c r="B21" s="2"/>
       <c r="C21" s="2"/>
       <c r="D21" s="4"/>
       <c r="E21" s="4"/>
-      <c r="F21" s="14"/>
+      <c r="F21" s="12"/>
       <c r="G21" s="8"/>
       <c r="H21" s="4"/>
       <c r="I21" s="4"/>
@@ -5852,7 +5962,7 @@
       <c r="C22" s="2"/>
       <c r="D22" s="4"/>
       <c r="E22" s="4"/>
-      <c r="F22" s="14"/>
+      <c r="F22" s="12"/>
       <c r="G22" s="8"/>
       <c r="H22" s="4"/>
       <c r="I22" s="4"/>
@@ -5864,24 +5974,13 @@
       <c r="C23" s="2"/>
       <c r="D23" s="4"/>
       <c r="E23" s="4"/>
-      <c r="F23" s="14"/>
+      <c r="F23" s="10"/>
       <c r="G23" s="8"/>
       <c r="H23" s="4"/>
       <c r="I23" s="4"/>
       <c r="J23" s="5"/>
     </row>
-    <row r="24" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="2"/>
-      <c r="B24" s="2"/>
-      <c r="C24" s="2"/>
-      <c r="D24" s="4"/>
-      <c r="E24" s="4"/>
-      <c r="F24" s="10"/>
-      <c r="G24" s="8"/>
-      <c r="H24" s="4"/>
-      <c r="I24" s="4"/>
-      <c r="J24" s="5"/>
-    </row>
+    <row r="24" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="25" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="26" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="27" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -6857,7 +6956,6 @@
     <row r="997" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="998" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="999" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="1000" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:J1"/>
@@ -6886,18 +6984,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="21" x14ac:dyDescent="0.35">
-      <c r="A1" s="12" t="s">
-        <v>440</v>
-      </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="13"/>
-      <c r="D1" s="13"/>
-      <c r="E1" s="13"/>
-      <c r="F1" s="13"/>
-      <c r="G1" s="13"/>
-      <c r="H1" s="13"/>
-      <c r="I1" s="13"/>
-      <c r="J1" s="13"/>
+      <c r="A1" s="16" t="s">
+        <v>412</v>
+      </c>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="17"/>
+      <c r="F1" s="17"/>
+      <c r="G1" s="17"/>
+      <c r="H1" s="17"/>
+      <c r="I1" s="17"/>
+      <c r="J1" s="17"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
@@ -6931,287 +7029,243 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:10" ht="88.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10" ht="136.5" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>441</v>
+        <v>414</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>447</v>
+        <v>413</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>10</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>453</v>
+        <v>421</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>448</v>
-      </c>
-      <c r="F3" s="14" t="s">
-        <v>454</v>
+        <v>420</v>
+      </c>
+      <c r="F3" s="12" t="s">
+        <v>427</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>50</v>
+        <v>258</v>
       </c>
       <c r="H3" s="4" t="s">
-        <v>455</v>
+        <v>434</v>
       </c>
       <c r="I3" s="4" t="s">
-        <v>488</v>
-      </c>
-      <c r="J3" s="5" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" ht="89.25" customHeight="1" x14ac:dyDescent="0.25">
+        <v>530</v>
+      </c>
+      <c r="J3" s="14" t="s">
+        <v>516</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" ht="91.5" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>442</v>
+        <v>415</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>447</v>
+        <v>413</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>40</v>
+        <v>10</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>456</v>
+        <v>422</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>448</v>
-      </c>
-      <c r="F4" s="14" t="s">
-        <v>457</v>
+        <v>420</v>
+      </c>
+      <c r="F4" s="12" t="s">
+        <v>428</v>
       </c>
       <c r="G4" s="8" t="s">
         <v>50</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>458</v>
-      </c>
-      <c r="I4" s="4"/>
-      <c r="J4" s="5"/>
-    </row>
-    <row r="5" spans="1:10" ht="85.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>435</v>
+      </c>
+      <c r="I4" s="4" t="s">
+        <v>531</v>
+      </c>
+      <c r="J4" s="14" t="s">
+        <v>516</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" ht="91.5" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>443</v>
+        <v>416</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>447</v>
+        <v>413</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>10</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>459</v>
+        <v>423</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>448</v>
-      </c>
-      <c r="F5" s="14" t="s">
-        <v>460</v>
+        <v>420</v>
+      </c>
+      <c r="F5" s="12" t="s">
+        <v>429</v>
       </c>
       <c r="G5" s="8" t="s">
-        <v>461</v>
+        <v>384</v>
       </c>
       <c r="H5" s="4" t="s">
-        <v>462</v>
-      </c>
-      <c r="I5" s="4"/>
-      <c r="J5" s="5"/>
-    </row>
-    <row r="6" spans="1:10" ht="79.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>436</v>
+      </c>
+      <c r="I5" s="4" t="s">
+        <v>533</v>
+      </c>
+      <c r="J5" s="14" t="s">
+        <v>516</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" ht="91.5" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>444</v>
+        <v>417</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>447</v>
+        <v>413</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>10</v>
+        <v>40</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>463</v>
+        <v>424</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>448</v>
-      </c>
-      <c r="F6" s="14" t="s">
-        <v>464</v>
+        <v>420</v>
+      </c>
+      <c r="F6" s="12" t="s">
+        <v>430</v>
       </c>
       <c r="G6" s="8" t="s">
-        <v>50</v>
+        <v>433</v>
       </c>
       <c r="H6" s="4" t="s">
-        <v>465</v>
-      </c>
-      <c r="I6" s="4"/>
-      <c r="J6" s="5"/>
-    </row>
-    <row r="7" spans="1:10" ht="81" customHeight="1" x14ac:dyDescent="0.25">
+        <v>437</v>
+      </c>
+      <c r="I6" s="4" t="s">
+        <v>534</v>
+      </c>
+      <c r="J6" s="14" t="s">
+        <v>516</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" ht="91.5" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>445</v>
+        <v>418</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>447</v>
+        <v>413</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>40</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>466</v>
+        <v>425</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>448</v>
-      </c>
-      <c r="F7" s="14" t="s">
-        <v>467</v>
+        <v>420</v>
+      </c>
+      <c r="F7" s="12" t="s">
+        <v>431</v>
       </c>
       <c r="G7" s="8" t="s">
-        <v>468</v>
+        <v>50</v>
       </c>
       <c r="H7" s="4" t="s">
-        <v>469</v>
-      </c>
-      <c r="I7" s="4"/>
-      <c r="J7" s="5"/>
-    </row>
-    <row r="8" spans="1:10" ht="76.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>438</v>
+      </c>
+      <c r="I7" s="4" t="s">
+        <v>535</v>
+      </c>
+      <c r="J7" s="14" t="s">
+        <v>516</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" ht="91.5" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>446</v>
+        <v>419</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>447</v>
+        <v>413</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>10</v>
+        <v>40</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>470</v>
+        <v>426</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>448</v>
-      </c>
-      <c r="F8" s="14" t="s">
-        <v>471</v>
+        <v>420</v>
+      </c>
+      <c r="F8" s="12" t="s">
+        <v>432</v>
       </c>
       <c r="G8" s="6" t="s">
         <v>50</v>
       </c>
       <c r="H8" s="4" t="s">
-        <v>472</v>
-      </c>
-      <c r="I8" s="4"/>
-      <c r="J8" s="5"/>
+        <v>439</v>
+      </c>
+      <c r="I8" s="4" t="s">
+        <v>532</v>
+      </c>
+      <c r="J8" s="14" t="s">
+        <v>516</v>
+      </c>
     </row>
     <row r="9" spans="1:10" ht="78" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="2" t="s">
-        <v>449</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>447</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="D9" s="4" t="s">
-        <v>473</v>
-      </c>
-      <c r="E9" s="4" t="s">
-        <v>448</v>
-      </c>
-      <c r="F9" s="14" t="s">
-        <v>474</v>
-      </c>
-      <c r="G9" s="8" t="s">
-        <v>50</v>
-      </c>
-      <c r="H9" s="4" t="s">
-        <v>475</v>
-      </c>
+      <c r="A9" s="2"/>
+      <c r="B9" s="2"/>
+      <c r="C9" s="2"/>
+      <c r="D9" s="4"/>
+      <c r="E9" s="4"/>
+      <c r="F9" s="12"/>
+      <c r="G9" s="8"/>
+      <c r="H9" s="4"/>
       <c r="I9" s="4"/>
       <c r="J9" s="5"/>
     </row>
     <row r="10" spans="1:10" ht="68.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="2" t="s">
-        <v>450</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>447</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="D10" s="4" t="s">
-        <v>476</v>
-      </c>
-      <c r="E10" s="4" t="s">
-        <v>448</v>
-      </c>
-      <c r="F10" s="14" t="s">
-        <v>477</v>
-      </c>
-      <c r="G10" s="8" t="s">
-        <v>50</v>
-      </c>
-      <c r="H10" s="4" t="s">
-        <v>478</v>
-      </c>
+      <c r="A10" s="2"/>
+      <c r="B10" s="2"/>
+      <c r="C10" s="2"/>
+      <c r="D10" s="4"/>
+      <c r="E10" s="4"/>
+      <c r="F10" s="12"/>
+      <c r="G10" s="8"/>
+      <c r="H10" s="4"/>
       <c r="I10" s="4"/>
       <c r="J10" s="5"/>
     </row>
     <row r="11" spans="1:10" ht="82.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="2" t="s">
-        <v>451</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>447</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="D11" s="4" t="s">
-        <v>479</v>
-      </c>
-      <c r="E11" s="4" t="s">
-        <v>448</v>
-      </c>
-      <c r="F11" s="14" t="s">
-        <v>480</v>
-      </c>
-      <c r="G11" s="8" t="s">
-        <v>50</v>
-      </c>
-      <c r="H11" s="4" t="s">
-        <v>481</v>
-      </c>
+      <c r="A11" s="2"/>
+      <c r="B11" s="2"/>
+      <c r="C11" s="2"/>
+      <c r="D11" s="4"/>
+      <c r="E11" s="4"/>
+      <c r="F11" s="12"/>
+      <c r="G11" s="8"/>
+      <c r="H11" s="4"/>
       <c r="I11" s="4"/>
       <c r="J11" s="5"/>
     </row>
     <row r="12" spans="1:10" ht="85.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="2" t="s">
-        <v>452</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>447</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="D12" s="4" t="s">
-        <v>482</v>
-      </c>
-      <c r="E12" s="4" t="s">
-        <v>448</v>
-      </c>
-      <c r="F12" s="14" t="s">
-        <v>483</v>
-      </c>
-      <c r="G12" s="8" t="s">
-        <v>50</v>
-      </c>
-      <c r="H12" s="4" t="s">
-        <v>484</v>
-      </c>
+      <c r="A12" s="2"/>
+      <c r="B12" s="2"/>
+      <c r="C12" s="2"/>
+      <c r="D12" s="4"/>
+      <c r="E12" s="4"/>
+      <c r="F12" s="12"/>
+      <c r="G12" s="8"/>
+      <c r="H12" s="4"/>
       <c r="I12" s="4"/>
       <c r="J12" s="5"/>
     </row>
@@ -7221,7 +7275,7 @@
       <c r="C13" s="2"/>
       <c r="D13" s="4"/>
       <c r="E13" s="4"/>
-      <c r="F13" s="14"/>
+      <c r="F13" s="12"/>
       <c r="G13" s="8"/>
       <c r="H13" s="4"/>
       <c r="I13" s="4"/>
@@ -7233,7 +7287,7 @@
       <c r="C14" s="2"/>
       <c r="D14" s="4"/>
       <c r="E14" s="4"/>
-      <c r="F14" s="14"/>
+      <c r="F14" s="12"/>
       <c r="G14" s="8"/>
       <c r="H14" s="4"/>
       <c r="I14" s="4"/>
@@ -7245,7 +7299,7 @@
       <c r="C15" s="2"/>
       <c r="D15" s="4"/>
       <c r="E15" s="4"/>
-      <c r="F15" s="14"/>
+      <c r="F15" s="12"/>
       <c r="G15" s="8"/>
       <c r="H15" s="4"/>
       <c r="I15" s="4"/>
@@ -7257,7 +7311,7 @@
       <c r="C16" s="2"/>
       <c r="D16" s="4"/>
       <c r="E16" s="4"/>
-      <c r="F16" s="14"/>
+      <c r="F16" s="12"/>
       <c r="G16" s="8"/>
       <c r="H16" s="4"/>
       <c r="I16" s="4"/>
@@ -7269,7 +7323,7 @@
       <c r="C17" s="2"/>
       <c r="D17" s="4"/>
       <c r="E17" s="4"/>
-      <c r="F17" s="14"/>
+      <c r="F17" s="12"/>
       <c r="G17" s="8"/>
       <c r="H17" s="4"/>
       <c r="I17" s="4"/>
@@ -7281,7 +7335,7 @@
       <c r="C18" s="2"/>
       <c r="D18" s="4"/>
       <c r="E18" s="4"/>
-      <c r="F18" s="14"/>
+      <c r="F18" s="12"/>
       <c r="G18" s="8"/>
       <c r="H18" s="4"/>
       <c r="I18" s="4"/>
@@ -7293,7 +7347,7 @@
       <c r="C19" s="2"/>
       <c r="D19" s="4"/>
       <c r="E19" s="4"/>
-      <c r="F19" s="14"/>
+      <c r="F19" s="12"/>
       <c r="G19" s="8"/>
       <c r="H19" s="4"/>
       <c r="I19" s="4"/>
@@ -7305,7 +7359,7 @@
       <c r="C20" s="2"/>
       <c r="D20" s="4"/>
       <c r="E20" s="4"/>
-      <c r="F20" s="14"/>
+      <c r="F20" s="12"/>
       <c r="G20" s="8"/>
       <c r="H20" s="4"/>
       <c r="I20" s="4"/>
@@ -7317,7 +7371,7 @@
       <c r="C21" s="2"/>
       <c r="D21" s="4"/>
       <c r="E21" s="4"/>
-      <c r="F21" s="14"/>
+      <c r="F21" s="12"/>
       <c r="G21" s="8"/>
       <c r="H21" s="4"/>
       <c r="I21" s="4"/>
@@ -7329,7 +7383,7 @@
       <c r="C22" s="2"/>
       <c r="D22" s="4"/>
       <c r="E22" s="4"/>
-      <c r="F22" s="14"/>
+      <c r="F22" s="12"/>
       <c r="G22" s="8"/>
       <c r="H22" s="4"/>
       <c r="I22" s="4"/>
@@ -7341,7 +7395,7 @@
       <c r="C23" s="2"/>
       <c r="D23" s="4"/>
       <c r="E23" s="4"/>
-      <c r="F23" s="14"/>
+      <c r="F23" s="12"/>
       <c r="G23" s="8"/>
       <c r="H23" s="4"/>
       <c r="I23" s="4"/>
@@ -8363,18 +8417,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="21" x14ac:dyDescent="0.35">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="16" t="s">
         <v>108</v>
       </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="13"/>
-      <c r="D1" s="13"/>
-      <c r="E1" s="13"/>
-      <c r="F1" s="13"/>
-      <c r="G1" s="13"/>
-      <c r="H1" s="13"/>
-      <c r="I1" s="13"/>
-      <c r="J1" s="13"/>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="17"/>
+      <c r="F1" s="17"/>
+      <c r="G1" s="17"/>
+      <c r="H1" s="17"/>
+      <c r="I1" s="17"/>
+      <c r="J1" s="17"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
@@ -8424,17 +8478,17 @@
       <c r="E3" s="4" t="s">
         <v>112</v>
       </c>
-      <c r="F3" s="14" t="s">
+      <c r="F3" s="12" t="s">
         <v>135</v>
       </c>
       <c r="G3" s="8" t="s">
         <v>113</v>
       </c>
       <c r="H3" s="4" t="s">
-        <v>492</v>
+        <v>486</v>
       </c>
       <c r="I3" s="4" t="s">
-        <v>488</v>
+        <v>482</v>
       </c>
       <c r="J3" s="5" t="s">
         <v>11</v>
@@ -8456,7 +8510,7 @@
       <c r="E4" s="4" t="s">
         <v>112</v>
       </c>
-      <c r="F4" s="14" t="s">
+      <c r="F4" s="12" t="s">
         <v>136</v>
       </c>
       <c r="G4" s="8" t="s">
@@ -8466,7 +8520,7 @@
         <v>116</v>
       </c>
       <c r="I4" s="4" t="s">
-        <v>493</v>
+        <v>487</v>
       </c>
       <c r="J4" s="5" t="s">
         <v>11</v>
@@ -8488,7 +8542,7 @@
       <c r="E5" s="4" t="s">
         <v>140</v>
       </c>
-      <c r="F5" s="14" t="s">
+      <c r="F5" s="12" t="s">
         <v>137</v>
       </c>
       <c r="G5" s="8" t="s">
@@ -8498,7 +8552,7 @@
         <v>119</v>
       </c>
       <c r="I5" s="4" t="s">
-        <v>493</v>
+        <v>487</v>
       </c>
       <c r="J5" s="5" t="s">
         <v>11</v>
@@ -8520,7 +8574,7 @@
       <c r="E6" s="4" t="s">
         <v>112</v>
       </c>
-      <c r="F6" s="14" t="s">
+      <c r="F6" s="12" t="s">
         <v>138</v>
       </c>
       <c r="G6" s="8" t="s">
@@ -8530,7 +8584,7 @@
         <v>123</v>
       </c>
       <c r="I6" s="4" t="s">
-        <v>488</v>
+        <v>482</v>
       </c>
       <c r="J6" s="5" t="s">
         <v>11</v>
@@ -8552,7 +8606,7 @@
       <c r="E7" s="4" t="s">
         <v>112</v>
       </c>
-      <c r="F7" s="14" t="s">
+      <c r="F7" s="12" t="s">
         <v>139</v>
       </c>
       <c r="G7" s="8" t="s">
@@ -8562,10 +8616,10 @@
         <v>141</v>
       </c>
       <c r="I7" s="4" t="s">
-        <v>488</v>
+        <v>482</v>
       </c>
       <c r="J7" s="5" t="s">
-        <v>486</v>
+        <v>480</v>
       </c>
     </row>
     <row r="8" spans="1:10" ht="76.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -8584,7 +8638,7 @@
       <c r="E8" s="4" t="s">
         <v>112</v>
       </c>
-      <c r="F8" s="14" t="s">
+      <c r="F8" s="12" t="s">
         <v>127</v>
       </c>
       <c r="G8" s="6" t="s">
@@ -8594,7 +8648,7 @@
         <v>128</v>
       </c>
       <c r="I8" s="4" t="s">
-        <v>488</v>
+        <v>482</v>
       </c>
       <c r="J8" s="5" t="s">
         <v>11</v>
@@ -8616,7 +8670,7 @@
       <c r="E9" s="4" t="s">
         <v>112</v>
       </c>
-      <c r="F9" s="14" t="s">
+      <c r="F9" s="12" t="s">
         <v>130</v>
       </c>
       <c r="G9" s="8" t="s">
@@ -8626,7 +8680,7 @@
         <v>131</v>
       </c>
       <c r="I9" s="4" t="s">
-        <v>488</v>
+        <v>482</v>
       </c>
       <c r="J9" s="5" t="s">
         <v>11</v>
@@ -8648,7 +8702,7 @@
       <c r="E10" s="4" t="s">
         <v>112</v>
       </c>
-      <c r="F10" s="14" t="s">
+      <c r="F10" s="12" t="s">
         <v>133</v>
       </c>
       <c r="G10" s="8" t="s">
@@ -8658,7 +8712,7 @@
         <v>134</v>
       </c>
       <c r="I10" s="4" t="s">
-        <v>488</v>
+        <v>482</v>
       </c>
       <c r="J10" s="5" t="s">
         <v>11</v>
@@ -8680,7 +8734,7 @@
       <c r="E11" s="4" t="s">
         <v>112</v>
       </c>
-      <c r="F11" s="14" t="s">
+      <c r="F11" s="12" t="s">
         <v>144</v>
       </c>
       <c r="G11" s="8" t="s">
@@ -8690,7 +8744,7 @@
         <v>145</v>
       </c>
       <c r="I11" s="4" t="s">
-        <v>488</v>
+        <v>482</v>
       </c>
       <c r="J11" s="5" t="s">
         <v>11</v>
@@ -8712,7 +8766,7 @@
       <c r="E12" s="4" t="s">
         <v>112</v>
       </c>
-      <c r="F12" s="14" t="s">
+      <c r="F12" s="12" t="s">
         <v>147</v>
       </c>
       <c r="G12" s="8" t="s">
@@ -8722,7 +8776,7 @@
         <v>149</v>
       </c>
       <c r="I12" s="4" t="s">
-        <v>488</v>
+        <v>482</v>
       </c>
       <c r="J12" s="5" t="s">
         <v>11</v>
@@ -8744,7 +8798,7 @@
       <c r="E13" s="4" t="s">
         <v>112</v>
       </c>
-      <c r="F13" s="14" t="s">
+      <c r="F13" s="12" t="s">
         <v>151</v>
       </c>
       <c r="G13" s="8" t="s">
@@ -8754,7 +8808,7 @@
         <v>153</v>
       </c>
       <c r="I13" s="4" t="s">
-        <v>488</v>
+        <v>482</v>
       </c>
       <c r="J13" s="5" t="s">
         <v>11</v>
@@ -8766,7 +8820,7 @@
       <c r="C14" s="2"/>
       <c r="D14" s="4"/>
       <c r="E14" s="4"/>
-      <c r="F14" s="14"/>
+      <c r="F14" s="12"/>
       <c r="G14" s="8"/>
       <c r="H14" s="4"/>
       <c r="I14" s="4"/>
@@ -8778,7 +8832,7 @@
       <c r="C15" s="2"/>
       <c r="D15" s="4"/>
       <c r="E15" s="4"/>
-      <c r="F15" s="14"/>
+      <c r="F15" s="12"/>
       <c r="G15" s="8"/>
       <c r="H15" s="4"/>
       <c r="I15" s="4"/>
@@ -8790,7 +8844,7 @@
       <c r="C16" s="2"/>
       <c r="D16" s="4"/>
       <c r="E16" s="4"/>
-      <c r="F16" s="14"/>
+      <c r="F16" s="12"/>
       <c r="G16" s="8"/>
       <c r="H16" s="4"/>
       <c r="I16" s="4"/>
@@ -8802,7 +8856,7 @@
       <c r="C17" s="2"/>
       <c r="D17" s="4"/>
       <c r="E17" s="4"/>
-      <c r="F17" s="14"/>
+      <c r="F17" s="12"/>
       <c r="G17" s="8"/>
       <c r="H17" s="4"/>
       <c r="I17" s="4"/>
@@ -8814,7 +8868,7 @@
       <c r="C18" s="2"/>
       <c r="D18" s="4"/>
       <c r="E18" s="4"/>
-      <c r="F18" s="14"/>
+      <c r="F18" s="12"/>
       <c r="G18" s="8"/>
       <c r="H18" s="4"/>
       <c r="I18" s="4"/>
@@ -8826,7 +8880,7 @@
       <c r="C19" s="2"/>
       <c r="D19" s="4"/>
       <c r="E19" s="4"/>
-      <c r="F19" s="14"/>
+      <c r="F19" s="12"/>
       <c r="G19" s="8"/>
       <c r="H19" s="4"/>
       <c r="I19" s="4"/>
@@ -8838,7 +8892,7 @@
       <c r="C20" s="2"/>
       <c r="D20" s="4"/>
       <c r="E20" s="4"/>
-      <c r="F20" s="14"/>
+      <c r="F20" s="12"/>
       <c r="G20" s="8"/>
       <c r="H20" s="4"/>
       <c r="I20" s="4"/>
@@ -8850,7 +8904,7 @@
       <c r="C21" s="2"/>
       <c r="D21" s="4"/>
       <c r="E21" s="4"/>
-      <c r="F21" s="14"/>
+      <c r="F21" s="12"/>
       <c r="G21" s="8"/>
       <c r="H21" s="4"/>
       <c r="I21" s="4"/>
@@ -8862,7 +8916,7 @@
       <c r="C22" s="2"/>
       <c r="D22" s="4"/>
       <c r="E22" s="4"/>
-      <c r="F22" s="14"/>
+      <c r="F22" s="12"/>
       <c r="G22" s="8"/>
       <c r="H22" s="4"/>
       <c r="I22" s="4"/>
@@ -8874,7 +8928,7 @@
       <c r="C23" s="2"/>
       <c r="D23" s="4"/>
       <c r="E23" s="4"/>
-      <c r="F23" s="14"/>
+      <c r="F23" s="12"/>
       <c r="G23" s="8"/>
       <c r="H23" s="4"/>
       <c r="I23" s="4"/>
@@ -9896,18 +9950,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="21" x14ac:dyDescent="0.35">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="16" t="s">
         <v>173</v>
       </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="13"/>
-      <c r="D1" s="13"/>
-      <c r="E1" s="13"/>
-      <c r="F1" s="13"/>
-      <c r="G1" s="13"/>
-      <c r="H1" s="13"/>
-      <c r="I1" s="13"/>
-      <c r="J1" s="13"/>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="17"/>
+      <c r="F1" s="17"/>
+      <c r="G1" s="17"/>
+      <c r="H1" s="17"/>
+      <c r="I1" s="17"/>
+      <c r="J1" s="17"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
@@ -9957,7 +10011,7 @@
       <c r="E3" s="4" t="s">
         <v>155</v>
       </c>
-      <c r="F3" s="14" t="s">
+      <c r="F3" s="12" t="s">
         <v>160</v>
       </c>
       <c r="G3" s="8" t="s">
@@ -9967,7 +10021,7 @@
         <v>162</v>
       </c>
       <c r="I3" s="4" t="s">
-        <v>488</v>
+        <v>482</v>
       </c>
       <c r="J3" s="5" t="s">
         <v>11</v>
@@ -9989,7 +10043,7 @@
       <c r="E4" s="4" t="s">
         <v>155</v>
       </c>
-      <c r="F4" s="14" t="s">
+      <c r="F4" s="12" t="s">
         <v>164</v>
       </c>
       <c r="G4" s="8" t="s">
@@ -9999,7 +10053,7 @@
         <v>165</v>
       </c>
       <c r="I4" s="4" t="s">
-        <v>488</v>
+        <v>482</v>
       </c>
       <c r="J4" s="5" t="s">
         <v>11</v>
@@ -10021,7 +10075,7 @@
       <c r="E5" s="4" t="s">
         <v>155</v>
       </c>
-      <c r="F5" s="14" t="s">
+      <c r="F5" s="12" t="s">
         <v>167</v>
       </c>
       <c r="G5" s="8" t="s">
@@ -10031,7 +10085,7 @@
         <v>169</v>
       </c>
       <c r="I5" s="4" t="s">
-        <v>488</v>
+        <v>482</v>
       </c>
       <c r="J5" s="5" t="s">
         <v>11</v>
@@ -10053,7 +10107,7 @@
       <c r="E6" s="4" t="s">
         <v>155</v>
       </c>
-      <c r="F6" s="14" t="s">
+      <c r="F6" s="12" t="s">
         <v>171</v>
       </c>
       <c r="G6" s="8" t="s">
@@ -10063,7 +10117,7 @@
         <v>172</v>
       </c>
       <c r="I6" s="4" t="s">
-        <v>488</v>
+        <v>482</v>
       </c>
       <c r="J6" s="5" t="s">
         <v>11</v>
@@ -10075,7 +10129,7 @@
       <c r="C7" s="2"/>
       <c r="D7" s="4"/>
       <c r="E7" s="4"/>
-      <c r="F7" s="14"/>
+      <c r="F7" s="12"/>
       <c r="G7" s="8"/>
       <c r="H7" s="4"/>
       <c r="I7" s="4"/>
@@ -10087,7 +10141,7 @@
       <c r="C8" s="2"/>
       <c r="D8" s="4"/>
       <c r="E8" s="4"/>
-      <c r="F8" s="14"/>
+      <c r="F8" s="12"/>
       <c r="G8" s="6"/>
       <c r="H8" s="4"/>
       <c r="I8" s="4"/>
@@ -10099,7 +10153,7 @@
       <c r="C9" s="2"/>
       <c r="D9" s="4"/>
       <c r="E9" s="4"/>
-      <c r="F9" s="14"/>
+      <c r="F9" s="12"/>
       <c r="G9" s="8"/>
       <c r="H9" s="4"/>
       <c r="I9" s="4"/>
@@ -10111,7 +10165,7 @@
       <c r="C10" s="2"/>
       <c r="D10" s="4"/>
       <c r="E10" s="4"/>
-      <c r="F10" s="14"/>
+      <c r="F10" s="12"/>
       <c r="G10" s="8"/>
       <c r="H10" s="4"/>
       <c r="I10" s="4"/>
@@ -10123,7 +10177,7 @@
       <c r="C11" s="2"/>
       <c r="D11" s="4"/>
       <c r="E11" s="4"/>
-      <c r="F11" s="14"/>
+      <c r="F11" s="12"/>
       <c r="G11" s="8"/>
       <c r="H11" s="4"/>
       <c r="I11" s="4"/>
@@ -10135,7 +10189,7 @@
       <c r="C12" s="2"/>
       <c r="D12" s="4"/>
       <c r="E12" s="4"/>
-      <c r="F12" s="14"/>
+      <c r="F12" s="12"/>
       <c r="G12" s="8"/>
       <c r="H12" s="4"/>
       <c r="I12" s="4"/>
@@ -10147,7 +10201,7 @@
       <c r="C13" s="2"/>
       <c r="D13" s="4"/>
       <c r="E13" s="4"/>
-      <c r="F13" s="14"/>
+      <c r="F13" s="12"/>
       <c r="G13" s="8"/>
       <c r="H13" s="4"/>
       <c r="I13" s="4"/>
@@ -10159,7 +10213,7 @@
       <c r="C14" s="2"/>
       <c r="D14" s="4"/>
       <c r="E14" s="4"/>
-      <c r="F14" s="14"/>
+      <c r="F14" s="12"/>
       <c r="G14" s="8"/>
       <c r="H14" s="4"/>
       <c r="I14" s="4"/>
@@ -10171,7 +10225,7 @@
       <c r="C15" s="2"/>
       <c r="D15" s="4"/>
       <c r="E15" s="4"/>
-      <c r="F15" s="14"/>
+      <c r="F15" s="12"/>
       <c r="G15" s="8"/>
       <c r="H15" s="4"/>
       <c r="I15" s="4"/>
@@ -10183,7 +10237,7 @@
       <c r="C16" s="2"/>
       <c r="D16" s="4"/>
       <c r="E16" s="4"/>
-      <c r="F16" s="14"/>
+      <c r="F16" s="12"/>
       <c r="G16" s="8"/>
       <c r="H16" s="4"/>
       <c r="I16" s="4"/>
@@ -10195,7 +10249,7 @@
       <c r="C17" s="2"/>
       <c r="D17" s="4"/>
       <c r="E17" s="4"/>
-      <c r="F17" s="14"/>
+      <c r="F17" s="12"/>
       <c r="G17" s="8"/>
       <c r="H17" s="4"/>
       <c r="I17" s="4"/>
@@ -10207,7 +10261,7 @@
       <c r="C18" s="2"/>
       <c r="D18" s="4"/>
       <c r="E18" s="4"/>
-      <c r="F18" s="14"/>
+      <c r="F18" s="12"/>
       <c r="G18" s="8"/>
       <c r="H18" s="4"/>
       <c r="I18" s="4"/>
@@ -10219,7 +10273,7 @@
       <c r="C19" s="2"/>
       <c r="D19" s="4"/>
       <c r="E19" s="4"/>
-      <c r="F19" s="14"/>
+      <c r="F19" s="12"/>
       <c r="G19" s="8"/>
       <c r="H19" s="4"/>
       <c r="I19" s="4"/>
@@ -10231,7 +10285,7 @@
       <c r="C20" s="2"/>
       <c r="D20" s="4"/>
       <c r="E20" s="4"/>
-      <c r="F20" s="14"/>
+      <c r="F20" s="12"/>
       <c r="G20" s="8"/>
       <c r="H20" s="4"/>
       <c r="I20" s="4"/>
@@ -10243,7 +10297,7 @@
       <c r="C21" s="2"/>
       <c r="D21" s="4"/>
       <c r="E21" s="4"/>
-      <c r="F21" s="14"/>
+      <c r="F21" s="12"/>
       <c r="G21" s="8"/>
       <c r="H21" s="4"/>
       <c r="I21" s="4"/>
@@ -10255,7 +10309,7 @@
       <c r="C22" s="2"/>
       <c r="D22" s="4"/>
       <c r="E22" s="4"/>
-      <c r="F22" s="14"/>
+      <c r="F22" s="12"/>
       <c r="G22" s="8"/>
       <c r="H22" s="4"/>
       <c r="I22" s="4"/>
@@ -10267,7 +10321,7 @@
       <c r="C23" s="2"/>
       <c r="D23" s="4"/>
       <c r="E23" s="4"/>
-      <c r="F23" s="14"/>
+      <c r="F23" s="12"/>
       <c r="G23" s="8"/>
       <c r="H23" s="4"/>
       <c r="I23" s="4"/>
@@ -11289,18 +11343,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="21" x14ac:dyDescent="0.35">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="16" t="s">
         <v>174</v>
       </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="13"/>
-      <c r="D1" s="13"/>
-      <c r="E1" s="13"/>
-      <c r="F1" s="13"/>
-      <c r="G1" s="13"/>
-      <c r="H1" s="13"/>
-      <c r="I1" s="13"/>
-      <c r="J1" s="13"/>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="17"/>
+      <c r="F1" s="17"/>
+      <c r="G1" s="17"/>
+      <c r="H1" s="17"/>
+      <c r="I1" s="17"/>
+      <c r="J1" s="17"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
@@ -11350,7 +11404,7 @@
       <c r="E3" s="4" t="s">
         <v>180</v>
       </c>
-      <c r="F3" s="14" t="s">
+      <c r="F3" s="12" t="s">
         <v>181</v>
       </c>
       <c r="G3" s="8" t="s">
@@ -11360,10 +11414,10 @@
         <v>184</v>
       </c>
       <c r="I3" s="4" t="s">
-        <v>523</v>
-      </c>
-      <c r="J3" s="16" t="s">
-        <v>522</v>
+        <v>517</v>
+      </c>
+      <c r="J3" s="14" t="s">
+        <v>516</v>
       </c>
     </row>
     <row r="4" spans="1:10" ht="89.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -11382,7 +11436,7 @@
       <c r="E4" s="4" t="s">
         <v>180</v>
       </c>
-      <c r="F4" s="14" t="s">
+      <c r="F4" s="12" t="s">
         <v>188</v>
       </c>
       <c r="G4" s="8" t="s">
@@ -11392,7 +11446,7 @@
         <v>187</v>
       </c>
       <c r="I4" s="4" t="s">
-        <v>488</v>
+        <v>482</v>
       </c>
       <c r="J4" s="5" t="s">
         <v>11</v>
@@ -11414,7 +11468,7 @@
       <c r="E5" s="4" t="s">
         <v>180</v>
       </c>
-      <c r="F5" s="14" t="s">
+      <c r="F5" s="12" t="s">
         <v>190</v>
       </c>
       <c r="G5" s="8" t="s">
@@ -11424,7 +11478,7 @@
         <v>191</v>
       </c>
       <c r="I5" s="4" t="s">
-        <v>488</v>
+        <v>482</v>
       </c>
       <c r="J5" s="5" t="s">
         <v>11</v>
@@ -11446,7 +11500,7 @@
       <c r="E6" s="4" t="s">
         <v>180</v>
       </c>
-      <c r="F6" s="14" t="s">
+      <c r="F6" s="12" t="s">
         <v>192</v>
       </c>
       <c r="G6" s="8" t="s">
@@ -11456,7 +11510,7 @@
         <v>194</v>
       </c>
       <c r="I6" s="4" t="s">
-        <v>495</v>
+        <v>489</v>
       </c>
       <c r="J6" s="5" t="s">
         <v>11</v>
@@ -11478,7 +11532,7 @@
       <c r="E7" s="4" t="s">
         <v>180</v>
       </c>
-      <c r="F7" s="14" t="s">
+      <c r="F7" s="12" t="s">
         <v>196</v>
       </c>
       <c r="G7" s="8" t="s">
@@ -11488,7 +11542,7 @@
         <v>197</v>
       </c>
       <c r="I7" s="4" t="s">
-        <v>488</v>
+        <v>482</v>
       </c>
       <c r="J7" s="5" t="s">
         <v>11</v>
@@ -11510,7 +11564,7 @@
       <c r="E8" s="4" t="s">
         <v>180</v>
       </c>
-      <c r="F8" s="14" t="s">
+      <c r="F8" s="12" t="s">
         <v>199</v>
       </c>
       <c r="G8" s="6" t="s">
@@ -11520,7 +11574,7 @@
         <v>200</v>
       </c>
       <c r="I8" s="4" t="s">
-        <v>488</v>
+        <v>482</v>
       </c>
       <c r="J8" s="5" t="s">
         <v>11</v>
@@ -11532,7 +11586,7 @@
       <c r="C9" s="2"/>
       <c r="D9" s="4"/>
       <c r="E9" s="4"/>
-      <c r="F9" s="14"/>
+      <c r="F9" s="12"/>
       <c r="G9" s="8"/>
       <c r="H9" s="4"/>
       <c r="I9" s="4"/>
@@ -11544,7 +11598,7 @@
       <c r="C10" s="2"/>
       <c r="D10" s="4"/>
       <c r="E10" s="4"/>
-      <c r="F10" s="14"/>
+      <c r="F10" s="12"/>
       <c r="G10" s="8"/>
       <c r="H10" s="4"/>
       <c r="I10" s="4"/>
@@ -11556,7 +11610,7 @@
       <c r="C11" s="2"/>
       <c r="D11" s="4"/>
       <c r="E11" s="4"/>
-      <c r="F11" s="14"/>
+      <c r="F11" s="12"/>
       <c r="G11" s="8"/>
       <c r="H11" s="4"/>
       <c r="I11" s="4"/>
@@ -11568,7 +11622,7 @@
       <c r="C12" s="2"/>
       <c r="D12" s="4"/>
       <c r="E12" s="4"/>
-      <c r="F12" s="14"/>
+      <c r="F12" s="12"/>
       <c r="G12" s="8"/>
       <c r="H12" s="4"/>
       <c r="I12" s="4"/>
@@ -11580,7 +11634,7 @@
       <c r="C13" s="2"/>
       <c r="D13" s="4"/>
       <c r="E13" s="4"/>
-      <c r="F13" s="14"/>
+      <c r="F13" s="12"/>
       <c r="G13" s="8"/>
       <c r="H13" s="4"/>
       <c r="I13" s="4"/>
@@ -11592,7 +11646,7 @@
       <c r="C14" s="2"/>
       <c r="D14" s="4"/>
       <c r="E14" s="4"/>
-      <c r="F14" s="14"/>
+      <c r="F14" s="12"/>
       <c r="G14" s="8"/>
       <c r="H14" s="4"/>
       <c r="I14" s="4"/>
@@ -11604,7 +11658,7 @@
       <c r="C15" s="2"/>
       <c r="D15" s="4"/>
       <c r="E15" s="4"/>
-      <c r="F15" s="14"/>
+      <c r="F15" s="12"/>
       <c r="G15" s="8"/>
       <c r="H15" s="4"/>
       <c r="I15" s="4"/>
@@ -11616,7 +11670,7 @@
       <c r="C16" s="2"/>
       <c r="D16" s="4"/>
       <c r="E16" s="4"/>
-      <c r="F16" s="14"/>
+      <c r="F16" s="12"/>
       <c r="G16" s="8"/>
       <c r="H16" s="4"/>
       <c r="I16" s="4"/>
@@ -11628,7 +11682,7 @@
       <c r="C17" s="2"/>
       <c r="D17" s="4"/>
       <c r="E17" s="4"/>
-      <c r="F17" s="14"/>
+      <c r="F17" s="12"/>
       <c r="G17" s="8"/>
       <c r="H17" s="4"/>
       <c r="I17" s="4"/>
@@ -11640,7 +11694,7 @@
       <c r="C18" s="2"/>
       <c r="D18" s="4"/>
       <c r="E18" s="4"/>
-      <c r="F18" s="14"/>
+      <c r="F18" s="12"/>
       <c r="G18" s="8"/>
       <c r="H18" s="4"/>
       <c r="I18" s="4"/>
@@ -11652,7 +11706,7 @@
       <c r="C19" s="2"/>
       <c r="D19" s="4"/>
       <c r="E19" s="4"/>
-      <c r="F19" s="14"/>
+      <c r="F19" s="12"/>
       <c r="G19" s="8"/>
       <c r="H19" s="4"/>
       <c r="I19" s="4"/>
@@ -11664,7 +11718,7 @@
       <c r="C20" s="2"/>
       <c r="D20" s="4"/>
       <c r="E20" s="4"/>
-      <c r="F20" s="14"/>
+      <c r="F20" s="12"/>
       <c r="G20" s="8"/>
       <c r="H20" s="4"/>
       <c r="I20" s="4"/>
@@ -11676,7 +11730,7 @@
       <c r="C21" s="2"/>
       <c r="D21" s="4"/>
       <c r="E21" s="4"/>
-      <c r="F21" s="14"/>
+      <c r="F21" s="12"/>
       <c r="G21" s="8"/>
       <c r="H21" s="4"/>
       <c r="I21" s="4"/>
@@ -11688,7 +11742,7 @@
       <c r="C22" s="2"/>
       <c r="D22" s="4"/>
       <c r="E22" s="4"/>
-      <c r="F22" s="14"/>
+      <c r="F22" s="12"/>
       <c r="G22" s="8"/>
       <c r="H22" s="4"/>
       <c r="I22" s="4"/>
@@ -11700,7 +11754,7 @@
       <c r="C23" s="2"/>
       <c r="D23" s="4"/>
       <c r="E23" s="4"/>
-      <c r="F23" s="14"/>
+      <c r="F23" s="12"/>
       <c r="G23" s="8"/>
       <c r="H23" s="4"/>
       <c r="I23" s="4"/>
@@ -12722,18 +12776,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="21" x14ac:dyDescent="0.35">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="16" t="s">
         <v>203</v>
       </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="13"/>
-      <c r="D1" s="13"/>
-      <c r="E1" s="13"/>
-      <c r="F1" s="13"/>
-      <c r="G1" s="13"/>
-      <c r="H1" s="13"/>
-      <c r="I1" s="13"/>
-      <c r="J1" s="13"/>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="17"/>
+      <c r="F1" s="17"/>
+      <c r="G1" s="17"/>
+      <c r="H1" s="17"/>
+      <c r="I1" s="17"/>
+      <c r="J1" s="17"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
@@ -12783,7 +12837,7 @@
       <c r="E3" s="4" t="s">
         <v>205</v>
       </c>
-      <c r="F3" s="14" t="s">
+      <c r="F3" s="12" t="s">
         <v>216</v>
       </c>
       <c r="G3" s="8" t="s">
@@ -12793,7 +12847,7 @@
         <v>218</v>
       </c>
       <c r="I3" s="4" t="s">
-        <v>488</v>
+        <v>482</v>
       </c>
       <c r="J3" s="5" t="s">
         <v>11</v>
@@ -12815,17 +12869,17 @@
       <c r="E4" s="4" t="s">
         <v>205</v>
       </c>
-      <c r="F4" s="14" t="s">
+      <c r="F4" s="12" t="s">
         <v>220</v>
       </c>
       <c r="G4" s="8" t="s">
         <v>221</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>496</v>
+        <v>490</v>
       </c>
       <c r="I4" s="4" t="s">
-        <v>488</v>
+        <v>482</v>
       </c>
       <c r="J4" s="5" t="s">
         <v>11</v>
@@ -12847,7 +12901,7 @@
       <c r="E5" s="4" t="s">
         <v>205</v>
       </c>
-      <c r="F5" s="14" t="s">
+      <c r="F5" s="12" t="s">
         <v>223</v>
       </c>
       <c r="G5" s="8" t="s">
@@ -12857,10 +12911,10 @@
         <v>224</v>
       </c>
       <c r="I5" s="4" t="s">
-        <v>497</v>
-      </c>
-      <c r="J5" s="15" t="s">
-        <v>494</v>
+        <v>491</v>
+      </c>
+      <c r="J5" s="13" t="s">
+        <v>488</v>
       </c>
     </row>
     <row r="6" spans="1:10" ht="79.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -12879,7 +12933,7 @@
       <c r="E6" s="4" t="s">
         <v>205</v>
       </c>
-      <c r="F6" s="14" t="s">
+      <c r="F6" s="12" t="s">
         <v>226</v>
       </c>
       <c r="G6" s="8" t="s">
@@ -12889,7 +12943,7 @@
         <v>228</v>
       </c>
       <c r="I6" s="4" t="s">
-        <v>488</v>
+        <v>482</v>
       </c>
       <c r="J6" s="5" t="s">
         <v>11</v>
@@ -12911,7 +12965,7 @@
       <c r="E7" s="4" t="s">
         <v>205</v>
       </c>
-      <c r="F7" s="14" t="s">
+      <c r="F7" s="12" t="s">
         <v>230</v>
       </c>
       <c r="G7" s="8" t="s">
@@ -12921,7 +12975,7 @@
         <v>232</v>
       </c>
       <c r="I7" s="4" t="s">
-        <v>488</v>
+        <v>482</v>
       </c>
       <c r="J7" s="5" t="s">
         <v>11</v>
@@ -12943,7 +12997,7 @@
       <c r="E8" s="4" t="s">
         <v>205</v>
       </c>
-      <c r="F8" s="14" t="s">
+      <c r="F8" s="12" t="s">
         <v>234</v>
       </c>
       <c r="G8" s="6" t="s">
@@ -12953,7 +13007,7 @@
         <v>236</v>
       </c>
       <c r="I8" s="4" t="s">
-        <v>488</v>
+        <v>482</v>
       </c>
       <c r="J8" s="5" t="s">
         <v>11</v>
@@ -12975,7 +13029,7 @@
       <c r="E9" s="4" t="s">
         <v>205</v>
       </c>
-      <c r="F9" s="14" t="s">
+      <c r="F9" s="12" t="s">
         <v>238</v>
       </c>
       <c r="G9" s="8" t="s">
@@ -12985,7 +13039,7 @@
         <v>240</v>
       </c>
       <c r="I9" s="4" t="s">
-        <v>488</v>
+        <v>482</v>
       </c>
       <c r="J9" s="5" t="s">
         <v>11</v>
@@ -13007,7 +13061,7 @@
       <c r="E10" s="4" t="s">
         <v>205</v>
       </c>
-      <c r="F10" s="14" t="s">
+      <c r="F10" s="12" t="s">
         <v>242</v>
       </c>
       <c r="G10" s="8" t="s">
@@ -13017,7 +13071,7 @@
         <v>244</v>
       </c>
       <c r="I10" s="4" t="s">
-        <v>498</v>
+        <v>492</v>
       </c>
       <c r="J10" s="5" t="s">
         <v>11</v>
@@ -13039,7 +13093,7 @@
       <c r="E11" s="4" t="s">
         <v>205</v>
       </c>
-      <c r="F11" s="14" t="s">
+      <c r="F11" s="12" t="s">
         <v>246</v>
       </c>
       <c r="G11" s="8" t="s">
@@ -13049,7 +13103,7 @@
         <v>247</v>
       </c>
       <c r="I11" s="4" t="s">
-        <v>488</v>
+        <v>482</v>
       </c>
       <c r="J11" s="5" t="s">
         <v>11</v>
@@ -13061,7 +13115,7 @@
       <c r="C12" s="2"/>
       <c r="D12" s="4"/>
       <c r="E12" s="4"/>
-      <c r="F12" s="14"/>
+      <c r="F12" s="12"/>
       <c r="G12" s="8"/>
       <c r="H12" s="4"/>
       <c r="I12" s="4"/>
@@ -13073,7 +13127,7 @@
       <c r="C13" s="2"/>
       <c r="D13" s="4"/>
       <c r="E13" s="4"/>
-      <c r="F13" s="14"/>
+      <c r="F13" s="12"/>
       <c r="G13" s="8"/>
       <c r="H13" s="4"/>
       <c r="I13" s="4"/>
@@ -13085,7 +13139,7 @@
       <c r="C14" s="2"/>
       <c r="D14" s="4"/>
       <c r="E14" s="4"/>
-      <c r="F14" s="14"/>
+      <c r="F14" s="12"/>
       <c r="G14" s="8"/>
       <c r="H14" s="4"/>
       <c r="I14" s="4"/>
@@ -13097,7 +13151,7 @@
       <c r="C15" s="2"/>
       <c r="D15" s="4"/>
       <c r="E15" s="4"/>
-      <c r="F15" s="14"/>
+      <c r="F15" s="12"/>
       <c r="G15" s="8"/>
       <c r="H15" s="4"/>
       <c r="I15" s="4"/>
@@ -13109,7 +13163,7 @@
       <c r="C16" s="2"/>
       <c r="D16" s="4"/>
       <c r="E16" s="4"/>
-      <c r="F16" s="14"/>
+      <c r="F16" s="12"/>
       <c r="G16" s="8"/>
       <c r="H16" s="4"/>
       <c r="I16" s="4"/>
@@ -13121,7 +13175,7 @@
       <c r="C17" s="2"/>
       <c r="D17" s="4"/>
       <c r="E17" s="4"/>
-      <c r="F17" s="14"/>
+      <c r="F17" s="12"/>
       <c r="G17" s="8"/>
       <c r="H17" s="4"/>
       <c r="I17" s="4"/>
@@ -13133,7 +13187,7 @@
       <c r="C18" s="2"/>
       <c r="D18" s="4"/>
       <c r="E18" s="4"/>
-      <c r="F18" s="14"/>
+      <c r="F18" s="12"/>
       <c r="G18" s="8"/>
       <c r="H18" s="4"/>
       <c r="I18" s="4"/>
@@ -13145,7 +13199,7 @@
       <c r="C19" s="2"/>
       <c r="D19" s="4"/>
       <c r="E19" s="4"/>
-      <c r="F19" s="14"/>
+      <c r="F19" s="12"/>
       <c r="G19" s="8"/>
       <c r="H19" s="4"/>
       <c r="I19" s="4"/>
@@ -13157,7 +13211,7 @@
       <c r="C20" s="2"/>
       <c r="D20" s="4"/>
       <c r="E20" s="4"/>
-      <c r="F20" s="14"/>
+      <c r="F20" s="12"/>
       <c r="G20" s="8"/>
       <c r="H20" s="4"/>
       <c r="I20" s="4"/>
@@ -13169,7 +13223,7 @@
       <c r="C21" s="2"/>
       <c r="D21" s="4"/>
       <c r="E21" s="4"/>
-      <c r="F21" s="14"/>
+      <c r="F21" s="12"/>
       <c r="G21" s="8"/>
       <c r="H21" s="4"/>
       <c r="I21" s="4"/>
@@ -13181,7 +13235,7 @@
       <c r="C22" s="2"/>
       <c r="D22" s="4"/>
       <c r="E22" s="4"/>
-      <c r="F22" s="14"/>
+      <c r="F22" s="12"/>
       <c r="G22" s="8"/>
       <c r="H22" s="4"/>
       <c r="I22" s="4"/>
@@ -13193,7 +13247,7 @@
       <c r="C23" s="2"/>
       <c r="D23" s="4"/>
       <c r="E23" s="4"/>
-      <c r="F23" s="14"/>
+      <c r="F23" s="12"/>
       <c r="G23" s="8"/>
       <c r="H23" s="4"/>
       <c r="I23" s="4"/>
@@ -14215,18 +14269,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="21" x14ac:dyDescent="0.35">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="16" t="s">
         <v>278</v>
       </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="13"/>
-      <c r="D1" s="13"/>
-      <c r="E1" s="13"/>
-      <c r="F1" s="13"/>
-      <c r="G1" s="13"/>
-      <c r="H1" s="13"/>
-      <c r="I1" s="13"/>
-      <c r="J1" s="13"/>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="17"/>
+      <c r="F1" s="17"/>
+      <c r="G1" s="17"/>
+      <c r="H1" s="17"/>
+      <c r="I1" s="17"/>
+      <c r="J1" s="17"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
@@ -14276,7 +14330,7 @@
       <c r="E3" s="4" t="s">
         <v>155</v>
       </c>
-      <c r="F3" s="14" t="s">
+      <c r="F3" s="12" t="s">
         <v>257</v>
       </c>
       <c r="G3" s="8" t="s">
@@ -14286,7 +14340,7 @@
         <v>259</v>
       </c>
       <c r="I3" s="4" t="s">
-        <v>499</v>
+        <v>493</v>
       </c>
       <c r="J3" s="5" t="s">
         <v>11</v>
@@ -14308,7 +14362,7 @@
       <c r="E4" s="4" t="s">
         <v>155</v>
       </c>
-      <c r="F4" s="14" t="s">
+      <c r="F4" s="12" t="s">
         <v>261</v>
       </c>
       <c r="G4" s="8" t="s">
@@ -14318,7 +14372,7 @@
         <v>264</v>
       </c>
       <c r="I4" s="4" t="s">
-        <v>488</v>
+        <v>482</v>
       </c>
       <c r="J4" s="5" t="s">
         <v>11</v>
@@ -14340,7 +14394,7 @@
       <c r="E5" s="4" t="s">
         <v>155</v>
       </c>
-      <c r="F5" s="14" t="s">
+      <c r="F5" s="12" t="s">
         <v>263</v>
       </c>
       <c r="G5" s="8" t="s">
@@ -14350,7 +14404,7 @@
         <v>266</v>
       </c>
       <c r="I5" s="4" t="s">
-        <v>488</v>
+        <v>482</v>
       </c>
       <c r="J5" s="5" t="s">
         <v>11</v>
@@ -14372,7 +14426,7 @@
       <c r="E6" s="4" t="s">
         <v>155</v>
       </c>
-      <c r="F6" s="14" t="s">
+      <c r="F6" s="12" t="s">
         <v>265</v>
       </c>
       <c r="G6" s="8" t="s">
@@ -14382,7 +14436,7 @@
         <v>267</v>
       </c>
       <c r="I6" s="4" t="s">
-        <v>488</v>
+        <v>482</v>
       </c>
       <c r="J6" s="5" t="s">
         <v>11</v>
@@ -14404,7 +14458,7 @@
       <c r="E7" s="4" t="s">
         <v>155</v>
       </c>
-      <c r="F7" s="14" t="s">
+      <c r="F7" s="12" t="s">
         <v>270</v>
       </c>
       <c r="G7" s="8" t="s">
@@ -14414,7 +14468,7 @@
         <v>271</v>
       </c>
       <c r="I7" s="4" t="s">
-        <v>488</v>
+        <v>482</v>
       </c>
       <c r="J7" s="5" t="s">
         <v>11</v>
@@ -14436,7 +14490,7 @@
       <c r="E8" s="4" t="s">
         <v>155</v>
       </c>
-      <c r="F8" s="14" t="s">
+      <c r="F8" s="12" t="s">
         <v>273</v>
       </c>
       <c r="G8" s="6" t="s">
@@ -14446,10 +14500,10 @@
         <v>274</v>
       </c>
       <c r="I8" s="4" t="s">
-        <v>500</v>
-      </c>
-      <c r="J8" s="15" t="s">
         <v>494</v>
+      </c>
+      <c r="J8" s="13" t="s">
+        <v>488</v>
       </c>
     </row>
     <row r="9" spans="1:10" ht="78" customHeight="1" x14ac:dyDescent="0.25">
@@ -14468,7 +14522,7 @@
       <c r="E9" s="4" t="s">
         <v>155</v>
       </c>
-      <c r="F9" s="14" t="s">
+      <c r="F9" s="12" t="s">
         <v>276</v>
       </c>
       <c r="G9" s="8" t="s">
@@ -14478,7 +14532,7 @@
         <v>277</v>
       </c>
       <c r="I9" s="4" t="s">
-        <v>501</v>
+        <v>495</v>
       </c>
       <c r="J9" s="5" t="s">
         <v>11</v>
@@ -14490,7 +14544,7 @@
       <c r="C10" s="2"/>
       <c r="D10" s="4"/>
       <c r="E10" s="4"/>
-      <c r="F10" s="14"/>
+      <c r="F10" s="12"/>
       <c r="G10" s="8"/>
       <c r="H10" s="4"/>
       <c r="I10" s="4"/>
@@ -14502,7 +14556,7 @@
       <c r="C11" s="2"/>
       <c r="D11" s="4"/>
       <c r="E11" s="4"/>
-      <c r="F11" s="14"/>
+      <c r="F11" s="12"/>
       <c r="G11" s="8"/>
       <c r="H11" s="4"/>
       <c r="I11" s="4"/>
@@ -14514,7 +14568,7 @@
       <c r="C12" s="2"/>
       <c r="D12" s="4"/>
       <c r="E12" s="4"/>
-      <c r="F12" s="14"/>
+      <c r="F12" s="12"/>
       <c r="G12" s="8"/>
       <c r="H12" s="4"/>
       <c r="I12" s="4"/>
@@ -14526,7 +14580,7 @@
       <c r="C13" s="2"/>
       <c r="D13" s="4"/>
       <c r="E13" s="4"/>
-      <c r="F13" s="14"/>
+      <c r="F13" s="12"/>
       <c r="G13" s="8"/>
       <c r="H13" s="4"/>
       <c r="I13" s="4"/>
@@ -14538,7 +14592,7 @@
       <c r="C14" s="2"/>
       <c r="D14" s="4"/>
       <c r="E14" s="4"/>
-      <c r="F14" s="14"/>
+      <c r="F14" s="12"/>
       <c r="G14" s="8"/>
       <c r="H14" s="4"/>
       <c r="I14" s="4"/>
@@ -14550,7 +14604,7 @@
       <c r="C15" s="2"/>
       <c r="D15" s="4"/>
       <c r="E15" s="4"/>
-      <c r="F15" s="14"/>
+      <c r="F15" s="12"/>
       <c r="G15" s="8"/>
       <c r="H15" s="4"/>
       <c r="I15" s="4"/>
@@ -14562,7 +14616,7 @@
       <c r="C16" s="2"/>
       <c r="D16" s="4"/>
       <c r="E16" s="4"/>
-      <c r="F16" s="14"/>
+      <c r="F16" s="12"/>
       <c r="G16" s="8"/>
       <c r="H16" s="4"/>
       <c r="I16" s="4"/>
@@ -14574,7 +14628,7 @@
       <c r="C17" s="2"/>
       <c r="D17" s="4"/>
       <c r="E17" s="4"/>
-      <c r="F17" s="14"/>
+      <c r="F17" s="12"/>
       <c r="G17" s="8"/>
       <c r="H17" s="4"/>
       <c r="I17" s="4"/>
@@ -14586,7 +14640,7 @@
       <c r="C18" s="2"/>
       <c r="D18" s="4"/>
       <c r="E18" s="4"/>
-      <c r="F18" s="14"/>
+      <c r="F18" s="12"/>
       <c r="G18" s="8"/>
       <c r="H18" s="4"/>
       <c r="I18" s="4"/>
@@ -14598,7 +14652,7 @@
       <c r="C19" s="2"/>
       <c r="D19" s="4"/>
       <c r="E19" s="4"/>
-      <c r="F19" s="14"/>
+      <c r="F19" s="12"/>
       <c r="G19" s="8"/>
       <c r="H19" s="4"/>
       <c r="I19" s="4"/>
@@ -14610,7 +14664,7 @@
       <c r="C20" s="2"/>
       <c r="D20" s="4"/>
       <c r="E20" s="4"/>
-      <c r="F20" s="14"/>
+      <c r="F20" s="12"/>
       <c r="G20" s="8"/>
       <c r="H20" s="4"/>
       <c r="I20" s="4"/>
@@ -14622,7 +14676,7 @@
       <c r="C21" s="2"/>
       <c r="D21" s="4"/>
       <c r="E21" s="4"/>
-      <c r="F21" s="14"/>
+      <c r="F21" s="12"/>
       <c r="G21" s="8"/>
       <c r="H21" s="4"/>
       <c r="I21" s="4"/>
@@ -14634,7 +14688,7 @@
       <c r="C22" s="2"/>
       <c r="D22" s="4"/>
       <c r="E22" s="4"/>
-      <c r="F22" s="14"/>
+      <c r="F22" s="12"/>
       <c r="G22" s="8"/>
       <c r="H22" s="4"/>
       <c r="I22" s="4"/>
@@ -14646,7 +14700,7 @@
       <c r="C23" s="2"/>
       <c r="D23" s="4"/>
       <c r="E23" s="4"/>
-      <c r="F23" s="14"/>
+      <c r="F23" s="12"/>
       <c r="G23" s="8"/>
       <c r="H23" s="4"/>
       <c r="I23" s="4"/>
@@ -15668,18 +15722,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="21" x14ac:dyDescent="0.35">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="16" t="s">
         <v>279</v>
       </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="13"/>
-      <c r="D1" s="13"/>
-      <c r="E1" s="13"/>
-      <c r="F1" s="13"/>
-      <c r="G1" s="13"/>
-      <c r="H1" s="13"/>
-      <c r="I1" s="13"/>
-      <c r="J1" s="13"/>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="17"/>
+      <c r="F1" s="17"/>
+      <c r="G1" s="17"/>
+      <c r="H1" s="17"/>
+      <c r="I1" s="17"/>
+      <c r="J1" s="17"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
@@ -15729,7 +15783,7 @@
       <c r="E3" s="4" t="s">
         <v>290</v>
       </c>
-      <c r="F3" s="14" t="s">
+      <c r="F3" s="12" t="s">
         <v>286</v>
       </c>
       <c r="G3" s="8" t="s">
@@ -15739,7 +15793,7 @@
         <v>287</v>
       </c>
       <c r="I3" s="4" t="s">
-        <v>488</v>
+        <v>482</v>
       </c>
       <c r="J3" s="5" t="s">
         <v>11</v>
@@ -15761,7 +15815,7 @@
       <c r="E4" s="4" t="s">
         <v>290</v>
       </c>
-      <c r="F4" s="14" t="s">
+      <c r="F4" s="12" t="s">
         <v>286</v>
       </c>
       <c r="G4" s="8" t="s">
@@ -15771,7 +15825,7 @@
         <v>289</v>
       </c>
       <c r="I4" s="4" t="s">
-        <v>488</v>
+        <v>482</v>
       </c>
       <c r="J4" s="5" t="s">
         <v>11</v>
@@ -15793,7 +15847,7 @@
       <c r="E5" s="4" t="s">
         <v>290</v>
       </c>
-      <c r="F5" s="14" t="s">
+      <c r="F5" s="12" t="s">
         <v>292</v>
       </c>
       <c r="G5" s="8" t="s">
@@ -15803,7 +15857,7 @@
         <v>293</v>
       </c>
       <c r="I5" s="4" t="s">
-        <v>488</v>
+        <v>482</v>
       </c>
       <c r="J5" s="5" t="s">
         <v>11</v>
@@ -15825,7 +15879,7 @@
       <c r="E6" s="4" t="s">
         <v>290</v>
       </c>
-      <c r="F6" s="14" t="s">
+      <c r="F6" s="12" t="s">
         <v>295</v>
       </c>
       <c r="G6" s="8" t="s">
@@ -15835,7 +15889,7 @@
         <v>296</v>
       </c>
       <c r="I6" s="4" t="s">
-        <v>488</v>
+        <v>482</v>
       </c>
       <c r="J6" s="5" t="s">
         <v>11</v>
@@ -15847,7 +15901,7 @@
       <c r="C7" s="2"/>
       <c r="D7" s="4"/>
       <c r="E7" s="4"/>
-      <c r="F7" s="14"/>
+      <c r="F7" s="12"/>
       <c r="G7" s="8"/>
       <c r="H7" s="4"/>
       <c r="I7" s="4"/>
@@ -15859,7 +15913,7 @@
       <c r="C8" s="2"/>
       <c r="D8" s="4"/>
       <c r="E8" s="4"/>
-      <c r="F8" s="14"/>
+      <c r="F8" s="12"/>
       <c r="G8" s="6"/>
       <c r="H8" s="4"/>
       <c r="I8" s="4"/>
@@ -15871,7 +15925,7 @@
       <c r="C9" s="2"/>
       <c r="D9" s="4"/>
       <c r="E9" s="4"/>
-      <c r="F9" s="14"/>
+      <c r="F9" s="12"/>
       <c r="G9" s="8"/>
       <c r="H9" s="4"/>
       <c r="I9" s="4"/>
@@ -15883,7 +15937,7 @@
       <c r="C10" s="2"/>
       <c r="D10" s="4"/>
       <c r="E10" s="4"/>
-      <c r="F10" s="14"/>
+      <c r="F10" s="12"/>
       <c r="G10" s="8"/>
       <c r="H10" s="4"/>
       <c r="I10" s="4"/>
@@ -15895,7 +15949,7 @@
       <c r="C11" s="2"/>
       <c r="D11" s="4"/>
       <c r="E11" s="4"/>
-      <c r="F11" s="14"/>
+      <c r="F11" s="12"/>
       <c r="G11" s="8"/>
       <c r="H11" s="4"/>
       <c r="I11" s="4"/>
@@ -15907,7 +15961,7 @@
       <c r="C12" s="2"/>
       <c r="D12" s="4"/>
       <c r="E12" s="4"/>
-      <c r="F12" s="14"/>
+      <c r="F12" s="12"/>
       <c r="G12" s="8"/>
       <c r="H12" s="4"/>
       <c r="I12" s="4"/>
@@ -15919,7 +15973,7 @@
       <c r="C13" s="2"/>
       <c r="D13" s="4"/>
       <c r="E13" s="4"/>
-      <c r="F13" s="14"/>
+      <c r="F13" s="12"/>
       <c r="G13" s="8"/>
       <c r="H13" s="4"/>
       <c r="I13" s="4"/>
@@ -15931,7 +15985,7 @@
       <c r="C14" s="2"/>
       <c r="D14" s="4"/>
       <c r="E14" s="4"/>
-      <c r="F14" s="14"/>
+      <c r="F14" s="12"/>
       <c r="G14" s="8"/>
       <c r="H14" s="4"/>
       <c r="I14" s="4"/>
@@ -15943,7 +15997,7 @@
       <c r="C15" s="2"/>
       <c r="D15" s="4"/>
       <c r="E15" s="4"/>
-      <c r="F15" s="14"/>
+      <c r="F15" s="12"/>
       <c r="G15" s="8"/>
       <c r="H15" s="4"/>
       <c r="I15" s="4"/>
@@ -15955,7 +16009,7 @@
       <c r="C16" s="2"/>
       <c r="D16" s="4"/>
       <c r="E16" s="4"/>
-      <c r="F16" s="14"/>
+      <c r="F16" s="12"/>
       <c r="G16" s="8"/>
       <c r="H16" s="4"/>
       <c r="I16" s="4"/>
@@ -15967,7 +16021,7 @@
       <c r="C17" s="2"/>
       <c r="D17" s="4"/>
       <c r="E17" s="4"/>
-      <c r="F17" s="14"/>
+      <c r="F17" s="12"/>
       <c r="G17" s="8"/>
       <c r="H17" s="4"/>
       <c r="I17" s="4"/>
@@ -15979,7 +16033,7 @@
       <c r="C18" s="2"/>
       <c r="D18" s="4"/>
       <c r="E18" s="4"/>
-      <c r="F18" s="14"/>
+      <c r="F18" s="12"/>
       <c r="G18" s="8"/>
       <c r="H18" s="4"/>
       <c r="I18" s="4"/>
@@ -15991,7 +16045,7 @@
       <c r="C19" s="2"/>
       <c r="D19" s="4"/>
       <c r="E19" s="4"/>
-      <c r="F19" s="14"/>
+      <c r="F19" s="12"/>
       <c r="G19" s="8"/>
       <c r="H19" s="4"/>
       <c r="I19" s="4"/>
@@ -16003,7 +16057,7 @@
       <c r="C20" s="2"/>
       <c r="D20" s="4"/>
       <c r="E20" s="4"/>
-      <c r="F20" s="14"/>
+      <c r="F20" s="12"/>
       <c r="G20" s="8"/>
       <c r="H20" s="4"/>
       <c r="I20" s="4"/>
@@ -16015,7 +16069,7 @@
       <c r="C21" s="2"/>
       <c r="D21" s="4"/>
       <c r="E21" s="4"/>
-      <c r="F21" s="14"/>
+      <c r="F21" s="12"/>
       <c r="G21" s="8"/>
       <c r="H21" s="4"/>
       <c r="I21" s="4"/>
@@ -16027,7 +16081,7 @@
       <c r="C22" s="2"/>
       <c r="D22" s="4"/>
       <c r="E22" s="4"/>
-      <c r="F22" s="14"/>
+      <c r="F22" s="12"/>
       <c r="G22" s="8"/>
       <c r="H22" s="4"/>
       <c r="I22" s="4"/>
@@ -16039,7 +16093,7 @@
       <c r="C23" s="2"/>
       <c r="D23" s="4"/>
       <c r="E23" s="4"/>
-      <c r="F23" s="14"/>
+      <c r="F23" s="12"/>
       <c r="G23" s="8"/>
       <c r="H23" s="4"/>
       <c r="I23" s="4"/>
@@ -17061,18 +17115,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="21" x14ac:dyDescent="0.35">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="16" t="s">
         <v>328</v>
       </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="13"/>
-      <c r="D1" s="13"/>
-      <c r="E1" s="13"/>
-      <c r="F1" s="13"/>
-      <c r="G1" s="13"/>
-      <c r="H1" s="13"/>
-      <c r="I1" s="13"/>
-      <c r="J1" s="13"/>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="17"/>
+      <c r="F1" s="17"/>
+      <c r="G1" s="17"/>
+      <c r="H1" s="17"/>
+      <c r="I1" s="17"/>
+      <c r="J1" s="17"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
@@ -17122,7 +17176,7 @@
       <c r="E3" s="4" t="s">
         <v>302</v>
       </c>
-      <c r="F3" s="14" t="s">
+      <c r="F3" s="12" t="s">
         <v>327</v>
       </c>
       <c r="G3" s="8" t="s">
@@ -17132,7 +17186,7 @@
         <v>308</v>
       </c>
       <c r="I3" s="4" t="s">
-        <v>488</v>
+        <v>482</v>
       </c>
       <c r="J3" s="5" t="s">
         <v>11</v>
@@ -17154,7 +17208,7 @@
       <c r="E4" s="4" t="s">
         <v>302</v>
       </c>
-      <c r="F4" s="14" t="s">
+      <c r="F4" s="12" t="s">
         <v>306</v>
       </c>
       <c r="G4" s="8" t="s">
@@ -17164,7 +17218,7 @@
         <v>309</v>
       </c>
       <c r="I4" s="4" t="s">
-        <v>488</v>
+        <v>482</v>
       </c>
       <c r="J4" s="5" t="s">
         <v>11</v>
@@ -17186,7 +17240,7 @@
       <c r="E5" s="4" t="s">
         <v>302</v>
       </c>
-      <c r="F5" s="14" t="s">
+      <c r="F5" s="12" t="s">
         <v>311</v>
       </c>
       <c r="G5" s="8" t="s">
@@ -17196,7 +17250,7 @@
         <v>313</v>
       </c>
       <c r="I5" s="4" t="s">
-        <v>488</v>
+        <v>482</v>
       </c>
       <c r="J5" s="5" t="s">
         <v>11</v>
@@ -17218,7 +17272,7 @@
       <c r="E6" s="4" t="s">
         <v>302</v>
       </c>
-      <c r="F6" s="14" t="s">
+      <c r="F6" s="12" t="s">
         <v>315</v>
       </c>
       <c r="G6" s="8" t="s">
@@ -17228,10 +17282,10 @@
         <v>322</v>
       </c>
       <c r="I6" s="4" t="s">
-        <v>502</v>
-      </c>
-      <c r="J6" s="15" t="s">
-        <v>494</v>
+        <v>496</v>
+      </c>
+      <c r="J6" s="13" t="s">
+        <v>488</v>
       </c>
     </row>
     <row r="7" spans="1:10" ht="81" customHeight="1" x14ac:dyDescent="0.25">
@@ -17250,17 +17304,17 @@
       <c r="E7" s="4" t="s">
         <v>302</v>
       </c>
-      <c r="F7" s="14" t="s">
+      <c r="F7" s="12" t="s">
         <v>320</v>
       </c>
       <c r="G7" s="8" t="s">
         <v>321</v>
       </c>
       <c r="H7" s="4" t="s">
-        <v>503</v>
+        <v>497</v>
       </c>
       <c r="I7" s="4" t="s">
-        <v>504</v>
+        <v>498</v>
       </c>
       <c r="J7" s="5" t="s">
         <v>11</v>
@@ -17282,7 +17336,7 @@
       <c r="E8" s="4" t="s">
         <v>302</v>
       </c>
-      <c r="F8" s="14" t="s">
+      <c r="F8" s="12" t="s">
         <v>324</v>
       </c>
       <c r="G8" s="6" t="s">
@@ -17292,10 +17346,10 @@
         <v>326</v>
       </c>
       <c r="I8" s="4" t="s">
-        <v>505</v>
-      </c>
-      <c r="J8" s="15" t="s">
-        <v>494</v>
+        <v>499</v>
+      </c>
+      <c r="J8" s="13" t="s">
+        <v>488</v>
       </c>
     </row>
     <row r="9" spans="1:10" ht="78" customHeight="1" x14ac:dyDescent="0.25">
@@ -17304,7 +17358,7 @@
       <c r="C9" s="2"/>
       <c r="D9" s="4"/>
       <c r="E9" s="4"/>
-      <c r="F9" s="14"/>
+      <c r="F9" s="12"/>
       <c r="G9" s="8"/>
       <c r="H9" s="4"/>
       <c r="I9" s="4"/>
@@ -17316,7 +17370,7 @@
       <c r="C10" s="2"/>
       <c r="D10" s="4"/>
       <c r="E10" s="4"/>
-      <c r="F10" s="14"/>
+      <c r="F10" s="12"/>
       <c r="G10" s="8"/>
       <c r="H10" s="4"/>
       <c r="I10" s="4"/>
@@ -17328,7 +17382,7 @@
       <c r="C11" s="2"/>
       <c r="D11" s="4"/>
       <c r="E11" s="4"/>
-      <c r="F11" s="14"/>
+      <c r="F11" s="12"/>
       <c r="G11" s="8"/>
       <c r="H11" s="4"/>
       <c r="I11" s="4"/>
@@ -17340,7 +17394,7 @@
       <c r="C12" s="2"/>
       <c r="D12" s="4"/>
       <c r="E12" s="4"/>
-      <c r="F12" s="14"/>
+      <c r="F12" s="12"/>
       <c r="G12" s="8"/>
       <c r="H12" s="4"/>
       <c r="I12" s="4"/>
@@ -17352,7 +17406,7 @@
       <c r="C13" s="2"/>
       <c r="D13" s="4"/>
       <c r="E13" s="4"/>
-      <c r="F13" s="14"/>
+      <c r="F13" s="12"/>
       <c r="G13" s="8"/>
       <c r="H13" s="4"/>
       <c r="I13" s="4"/>
@@ -17364,7 +17418,7 @@
       <c r="C14" s="2"/>
       <c r="D14" s="4"/>
       <c r="E14" s="4"/>
-      <c r="F14" s="14"/>
+      <c r="F14" s="12"/>
       <c r="G14" s="8"/>
       <c r="H14" s="4"/>
       <c r="I14" s="4"/>
@@ -17376,7 +17430,7 @@
       <c r="C15" s="2"/>
       <c r="D15" s="4"/>
       <c r="E15" s="4"/>
-      <c r="F15" s="14"/>
+      <c r="F15" s="12"/>
       <c r="G15" s="8"/>
       <c r="H15" s="4"/>
       <c r="I15" s="4"/>
@@ -17388,7 +17442,7 @@
       <c r="C16" s="2"/>
       <c r="D16" s="4"/>
       <c r="E16" s="4"/>
-      <c r="F16" s="14"/>
+      <c r="F16" s="12"/>
       <c r="G16" s="8"/>
       <c r="H16" s="4"/>
       <c r="I16" s="4"/>
@@ -17400,7 +17454,7 @@
       <c r="C17" s="2"/>
       <c r="D17" s="4"/>
       <c r="E17" s="4"/>
-      <c r="F17" s="14"/>
+      <c r="F17" s="12"/>
       <c r="G17" s="8"/>
       <c r="H17" s="4"/>
       <c r="I17" s="4"/>
@@ -17412,7 +17466,7 @@
       <c r="C18" s="2"/>
       <c r="D18" s="4"/>
       <c r="E18" s="4"/>
-      <c r="F18" s="14"/>
+      <c r="F18" s="12"/>
       <c r="G18" s="8"/>
       <c r="H18" s="4"/>
       <c r="I18" s="4"/>
@@ -17424,7 +17478,7 @@
       <c r="C19" s="2"/>
       <c r="D19" s="4"/>
       <c r="E19" s="4"/>
-      <c r="F19" s="14"/>
+      <c r="F19" s="12"/>
       <c r="G19" s="8"/>
       <c r="H19" s="4"/>
       <c r="I19" s="4"/>
@@ -17436,7 +17490,7 @@
       <c r="C20" s="2"/>
       <c r="D20" s="4"/>
       <c r="E20" s="4"/>
-      <c r="F20" s="14"/>
+      <c r="F20" s="12"/>
       <c r="G20" s="8"/>
       <c r="H20" s="4"/>
       <c r="I20" s="4"/>
@@ -17448,7 +17502,7 @@
       <c r="C21" s="2"/>
       <c r="D21" s="4"/>
       <c r="E21" s="4"/>
-      <c r="F21" s="14"/>
+      <c r="F21" s="12"/>
       <c r="G21" s="8"/>
       <c r="H21" s="4"/>
       <c r="I21" s="4"/>
@@ -17460,7 +17514,7 @@
       <c r="C22" s="2"/>
       <c r="D22" s="4"/>
       <c r="E22" s="4"/>
-      <c r="F22" s="14"/>
+      <c r="F22" s="12"/>
       <c r="G22" s="8"/>
       <c r="H22" s="4"/>
       <c r="I22" s="4"/>
@@ -17472,7 +17526,7 @@
       <c r="C23" s="2"/>
       <c r="D23" s="4"/>
       <c r="E23" s="4"/>
-      <c r="F23" s="14"/>
+      <c r="F23" s="12"/>
       <c r="G23" s="8"/>
       <c r="H23" s="4"/>
       <c r="I23" s="4"/>
@@ -18494,18 +18548,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="21" x14ac:dyDescent="0.35">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="16" t="s">
         <v>329</v>
       </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="13"/>
-      <c r="D1" s="13"/>
-      <c r="E1" s="13"/>
-      <c r="F1" s="13"/>
-      <c r="G1" s="13"/>
-      <c r="H1" s="13"/>
-      <c r="I1" s="13"/>
-      <c r="J1" s="13"/>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="17"/>
+      <c r="F1" s="17"/>
+      <c r="G1" s="17"/>
+      <c r="H1" s="17"/>
+      <c r="I1" s="17"/>
+      <c r="J1" s="17"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
@@ -18555,7 +18609,7 @@
       <c r="E3" s="4" t="s">
         <v>205</v>
       </c>
-      <c r="F3" s="14" t="s">
+      <c r="F3" s="12" t="s">
         <v>353</v>
       </c>
       <c r="G3" s="8" t="s">
@@ -18565,7 +18619,7 @@
         <v>354</v>
       </c>
       <c r="I3" s="4" t="s">
-        <v>488</v>
+        <v>482</v>
       </c>
       <c r="J3" s="5" t="s">
         <v>11</v>
@@ -18587,7 +18641,7 @@
       <c r="E4" s="4" t="s">
         <v>205</v>
       </c>
-      <c r="F4" s="14" t="s">
+      <c r="F4" s="12" t="s">
         <v>355</v>
       </c>
       <c r="G4" s="8" t="s">
@@ -18597,7 +18651,7 @@
         <v>356</v>
       </c>
       <c r="I4" s="4" t="s">
-        <v>488</v>
+        <v>482</v>
       </c>
       <c r="J4" s="5" t="s">
         <v>11</v>
@@ -18619,7 +18673,7 @@
       <c r="E5" s="4" t="s">
         <v>205</v>
       </c>
-      <c r="F5" s="14" t="s">
+      <c r="F5" s="12" t="s">
         <v>357</v>
       </c>
       <c r="G5" s="8" t="s">
@@ -18629,7 +18683,7 @@
         <v>358</v>
       </c>
       <c r="I5" s="4" t="s">
-        <v>488</v>
+        <v>482</v>
       </c>
       <c r="J5" s="5" t="s">
         <v>11</v>
@@ -18651,7 +18705,7 @@
       <c r="E6" s="4" t="s">
         <v>205</v>
       </c>
-      <c r="F6" s="14" t="s">
+      <c r="F6" s="12" t="s">
         <v>359</v>
       </c>
       <c r="G6" s="8" t="s">
@@ -18661,7 +18715,7 @@
         <v>368</v>
       </c>
       <c r="I6" s="4" t="s">
-        <v>488</v>
+        <v>482</v>
       </c>
       <c r="J6" s="5" t="s">
         <v>11</v>
@@ -18683,7 +18737,7 @@
       <c r="E7" s="4" t="s">
         <v>205</v>
       </c>
-      <c r="F7" s="14" t="s">
+      <c r="F7" s="12" t="s">
         <v>360</v>
       </c>
       <c r="G7" s="8" t="s">
@@ -18693,7 +18747,7 @@
         <v>361</v>
       </c>
       <c r="I7" s="4" t="s">
-        <v>488</v>
+        <v>482</v>
       </c>
       <c r="J7" s="5" t="s">
         <v>11</v>
@@ -18715,7 +18769,7 @@
       <c r="E8" s="4" t="s">
         <v>205</v>
       </c>
-      <c r="F8" s="14" t="s">
+      <c r="F8" s="12" t="s">
         <v>362</v>
       </c>
       <c r="G8" s="6" t="s">
@@ -18725,7 +18779,7 @@
         <v>363</v>
       </c>
       <c r="I8" s="4" t="s">
-        <v>488</v>
+        <v>482</v>
       </c>
       <c r="J8" s="5" t="s">
         <v>11</v>
@@ -18747,7 +18801,7 @@
       <c r="E9" s="4" t="s">
         <v>205</v>
       </c>
-      <c r="F9" s="14" t="s">
+      <c r="F9" s="12" t="s">
         <v>364</v>
       </c>
       <c r="G9" s="8" t="s">
@@ -18757,7 +18811,7 @@
         <v>366</v>
       </c>
       <c r="I9" s="4" t="s">
-        <v>488</v>
+        <v>482</v>
       </c>
       <c r="J9" s="5" t="s">
         <v>11</v>
@@ -18779,7 +18833,7 @@
       <c r="E10" s="4" t="s">
         <v>205</v>
       </c>
-      <c r="F10" s="14" t="s">
+      <c r="F10" s="12" t="s">
         <v>365</v>
       </c>
       <c r="G10" s="8" t="s">
@@ -18789,7 +18843,7 @@
         <v>367</v>
       </c>
       <c r="I10" s="4" t="s">
-        <v>488</v>
+        <v>482</v>
       </c>
       <c r="J10" s="5" t="s">
         <v>11</v>
@@ -18811,7 +18865,7 @@
       <c r="E11" s="4" t="s">
         <v>205</v>
       </c>
-      <c r="F11" s="14" t="s">
+      <c r="F11" s="12" t="s">
         <v>369</v>
       </c>
       <c r="G11" s="8" t="s">
@@ -18821,7 +18875,7 @@
         <v>370</v>
       </c>
       <c r="I11" s="4" t="s">
-        <v>488</v>
+        <v>482</v>
       </c>
       <c r="J11" s="5" t="s">
         <v>11</v>
@@ -18843,7 +18897,7 @@
       <c r="E12" s="4" t="s">
         <v>205</v>
       </c>
-      <c r="F12" s="14" t="s">
+      <c r="F12" s="12" t="s">
         <v>371</v>
       </c>
       <c r="G12" s="8" t="s">
@@ -18853,7 +18907,7 @@
         <v>372</v>
       </c>
       <c r="I12" s="4" t="s">
-        <v>488</v>
+        <v>482</v>
       </c>
       <c r="J12" s="5" t="s">
         <v>11</v>
@@ -18875,7 +18929,7 @@
       <c r="E13" s="4" t="s">
         <v>205</v>
       </c>
-      <c r="F13" s="14" t="s">
+      <c r="F13" s="12" t="s">
         <v>373</v>
       </c>
       <c r="G13" s="8" t="s">
@@ -18885,10 +18939,10 @@
         <v>374</v>
       </c>
       <c r="I13" s="4" t="s">
-        <v>525</v>
-      </c>
-      <c r="J13" s="17" t="s">
-        <v>524</v>
+        <v>519</v>
+      </c>
+      <c r="J13" s="15" t="s">
+        <v>518</v>
       </c>
     </row>
     <row r="14" spans="1:10" ht="88.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -18907,7 +18961,7 @@
       <c r="E14" s="4" t="s">
         <v>205</v>
       </c>
-      <c r="F14" s="14" t="s">
+      <c r="F14" s="12" t="s">
         <v>377</v>
       </c>
       <c r="G14" s="8" t="s">
@@ -18917,7 +18971,7 @@
         <v>378</v>
       </c>
       <c r="I14" s="4" t="s">
-        <v>488</v>
+        <v>482</v>
       </c>
       <c r="J14" s="5" t="s">
         <v>11</v>
@@ -18925,7 +18979,7 @@
     </row>
     <row r="15" spans="1:10" ht="73.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>515</v>
+        <v>509</v>
       </c>
       <c r="B15" s="2" t="s">
         <v>336</v>
@@ -18934,25 +18988,25 @@
         <v>40</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>514</v>
+        <v>508</v>
       </c>
       <c r="E15" s="4" t="s">
         <v>205</v>
       </c>
-      <c r="F15" s="14" t="s">
-        <v>516</v>
+      <c r="F15" s="12" t="s">
+        <v>510</v>
       </c>
       <c r="G15" s="8" t="s">
-        <v>517</v>
+        <v>511</v>
       </c>
       <c r="H15" s="4" t="s">
-        <v>518</v>
+        <v>512</v>
       </c>
       <c r="I15" s="4" t="s">
-        <v>519</v>
-      </c>
-      <c r="J15" s="15" t="s">
-        <v>494</v>
+        <v>513</v>
+      </c>
+      <c r="J15" s="13" t="s">
+        <v>488</v>
       </c>
     </row>
     <row r="16" spans="1:10" ht="75" customHeight="1" x14ac:dyDescent="0.25">
@@ -18961,7 +19015,7 @@
       <c r="C16" s="2"/>
       <c r="D16" s="4"/>
       <c r="E16" s="4"/>
-      <c r="F16" s="14"/>
+      <c r="F16" s="12"/>
       <c r="G16" s="8"/>
       <c r="H16" s="4"/>
       <c r="I16" s="4"/>
@@ -18973,7 +19027,7 @@
       <c r="C17" s="2"/>
       <c r="D17" s="4"/>
       <c r="E17" s="4"/>
-      <c r="F17" s="14"/>
+      <c r="F17" s="12"/>
       <c r="G17" s="8"/>
       <c r="H17" s="4"/>
       <c r="I17" s="4"/>
@@ -18985,7 +19039,7 @@
       <c r="C18" s="2"/>
       <c r="D18" s="4"/>
       <c r="E18" s="4"/>
-      <c r="F18" s="14"/>
+      <c r="F18" s="12"/>
       <c r="G18" s="8"/>
       <c r="H18" s="4"/>
       <c r="I18" s="4"/>
@@ -18997,7 +19051,7 @@
       <c r="C19" s="2"/>
       <c r="D19" s="4"/>
       <c r="E19" s="4"/>
-      <c r="F19" s="14"/>
+      <c r="F19" s="12"/>
       <c r="G19" s="8"/>
       <c r="H19" s="4"/>
       <c r="I19" s="4"/>
@@ -19009,7 +19063,7 @@
       <c r="C20" s="2"/>
       <c r="D20" s="4"/>
       <c r="E20" s="4"/>
-      <c r="F20" s="14"/>
+      <c r="F20" s="12"/>
       <c r="G20" s="8"/>
       <c r="H20" s="4"/>
       <c r="I20" s="4"/>
@@ -19021,7 +19075,7 @@
       <c r="C21" s="2"/>
       <c r="D21" s="4"/>
       <c r="E21" s="4"/>
-      <c r="F21" s="14"/>
+      <c r="F21" s="12"/>
       <c r="G21" s="8"/>
       <c r="H21" s="4"/>
       <c r="I21" s="4"/>
@@ -19033,7 +19087,7 @@
       <c r="C22" s="2"/>
       <c r="D22" s="4"/>
       <c r="E22" s="4"/>
-      <c r="F22" s="14"/>
+      <c r="F22" s="12"/>
       <c r="G22" s="8"/>
       <c r="H22" s="4"/>
       <c r="I22" s="4"/>
@@ -19045,7 +19099,7 @@
       <c r="C23" s="2"/>
       <c r="D23" s="4"/>
       <c r="E23" s="4"/>
-      <c r="F23" s="14"/>
+      <c r="F23" s="12"/>
       <c r="G23" s="8"/>
       <c r="H23" s="4"/>
       <c r="I23" s="4"/>

</xml_diff>